<commit_message>
Genislet: Fabrika Yerlesim Plani'nda tum 20 makine icin bransman cizimi
</commit_message>
<xml_diff>
--- a/dust_collection_tool.xlsx
+++ b/dust_collection_tool.xlsx
@@ -47,7 +47,7 @@
     <numFmt numFmtId="174" formatCode="#,##0 &quot;kWh&quot;"/>
     <numFmt numFmtId="175" formatCode="#,##0.0 &quot;m2&quot;"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="20">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -122,6 +122,11 @@
       <b val="1"/>
       <color rgb="001F3864"/>
       <sz val="13"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="7"/>
     </font>
     <font>
       <b val="1"/>
@@ -566,45 +571,45 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="169" fontId="18" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="169" fontId="19" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="18" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="170" fontId="19" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="171" fontId="18" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="171" fontId="19" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="18" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="172" fontId="19" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="18" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="173" fontId="19" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="174" fontId="18" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="174" fontId="19" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="175" fontId="18" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="175" fontId="19" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1134,9 +1139,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>5</col>
+      <col>53</col>
       <colOff>0</colOff>
-      <row>18</row>
+      <row>10</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="152400" cy="152400"/>
@@ -1159,9 +1164,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>13</col>
+      <col>61</col>
       <colOff>0</colOff>
-      <row>18</row>
+      <row>10</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="152400" cy="152400"/>
@@ -1184,9 +1189,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>21</col>
+      <col>69</col>
       <colOff>0</colOff>
-      <row>18</row>
+      <row>10</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="152400" cy="152400"/>
@@ -1209,9 +1214,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>29</col>
+      <col>77</col>
       <colOff>0</colOff>
-      <row>18</row>
+      <row>10</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="152400" cy="152400"/>
@@ -1234,7 +1239,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>37</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>18</row>
       <rowOff>0</rowOff>
@@ -1259,7 +1264,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>45</col>
+      <col>13</col>
       <colOff>0</colOff>
       <row>18</row>
       <rowOff>0</rowOff>
@@ -1284,9 +1289,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>5</col>
+      <col>21</col>
       <colOff>0</colOff>
-      <row>26</row>
+      <row>18</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="152400" cy="152400"/>
@@ -1309,9 +1314,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>13</col>
+      <col>29</col>
       <colOff>0</colOff>
-      <row>26</row>
+      <row>18</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="152400" cy="152400"/>
@@ -1334,9 +1339,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>21</col>
+      <col>37</col>
       <colOff>0</colOff>
-      <row>26</row>
+      <row>18</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="152400" cy="152400"/>
@@ -1359,9 +1364,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>29</col>
+      <col>45</col>
       <colOff>0</colOff>
-      <row>26</row>
+      <row>18</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="152400" cy="152400"/>
@@ -1384,9 +1389,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>37</col>
+      <col>53</col>
       <colOff>0</colOff>
-      <row>26</row>
+      <row>18</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="152400" cy="152400"/>
@@ -1409,9 +1414,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>45</col>
+      <col>61</col>
       <colOff>0</colOff>
-      <row>26</row>
+      <row>18</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="152400" cy="152400"/>
@@ -1434,9 +1439,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>5</col>
+      <col>69</col>
       <colOff>0</colOff>
-      <row>34</row>
+      <row>18</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="152400" cy="152400"/>
@@ -1459,9 +1464,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>13</col>
+      <col>77</col>
       <colOff>0</colOff>
-      <row>34</row>
+      <row>18</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="152400" cy="152400"/>
@@ -1484,9 +1489,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>21</col>
+      <col>5</col>
       <colOff>0</colOff>
-      <row>34</row>
+      <row>26</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="152400" cy="152400"/>
@@ -1509,9 +1514,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>29</col>
+      <col>13</col>
       <colOff>0</colOff>
-      <row>34</row>
+      <row>26</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="152400" cy="152400"/>
@@ -1534,9 +1539,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>37</col>
+      <col>21</col>
       <colOff>0</colOff>
-      <row>34</row>
+      <row>26</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="152400" cy="152400"/>
@@ -1559,9 +1564,9 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>45</col>
+      <col>29</col>
       <colOff>0</colOff>
-      <row>34</row>
+      <row>26</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="152400" cy="152400"/>
@@ -1584,12 +1589,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>10</col>
+      <col>37</col>
       <colOff>0</colOff>
-      <row>21</row>
+      <row>26</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="419100" cy="314325"/>
+    <ext cx="152400" cy="152400"/>
     <pic>
       <nvPicPr>
         <cNvPr id="25" name="Image 25" descr="Picture"/>
@@ -1609,12 +1614,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>22</col>
+      <col>45</col>
       <colOff>0</colOff>
-      <row>21</row>
+      <row>26</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="419100" cy="314325"/>
+    <ext cx="152400" cy="152400"/>
     <pic>
       <nvPicPr>
         <cNvPr id="26" name="Image 26" descr="Picture"/>
@@ -1634,12 +1639,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>34</col>
+      <col>53</col>
       <colOff>0</colOff>
-      <row>21</row>
+      <row>26</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="419100" cy="314325"/>
+    <ext cx="152400" cy="152400"/>
     <pic>
       <nvPicPr>
         <cNvPr id="27" name="Image 27" descr="Picture"/>
@@ -1647,6 +1652,831 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId27"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>61</col>
+      <colOff>0</colOff>
+      <row>26</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="152400" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="28" name="Image 28" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId28"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>69</col>
+      <colOff>0</colOff>
+      <row>26</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="152400" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="29" name="Image 29" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId29"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>77</col>
+      <colOff>0</colOff>
+      <row>26</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="152400" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="30" name="Image 30" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId30"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>34</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="152400" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="31" name="Image 31" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId31"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>13</col>
+      <colOff>0</colOff>
+      <row>34</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="152400" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="32" name="Image 32" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId32"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>21</col>
+      <colOff>0</colOff>
+      <row>34</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="152400" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="33" name="Image 33" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId33"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>29</col>
+      <colOff>0</colOff>
+      <row>34</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="152400" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="34" name="Image 34" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId34"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>37</col>
+      <colOff>0</colOff>
+      <row>34</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="152400" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="35" name="Image 35" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId35"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>45</col>
+      <colOff>0</colOff>
+      <row>34</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="152400" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="36" name="Image 36" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId36"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>53</col>
+      <colOff>0</colOff>
+      <row>34</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="152400" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="37" name="Image 37" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId37"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>61</col>
+      <colOff>0</colOff>
+      <row>34</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="152400" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="38" name="Image 38" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId38"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>69</col>
+      <colOff>0</colOff>
+      <row>34</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="152400" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="39" name="Image 39" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId39"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>77</col>
+      <colOff>0</colOff>
+      <row>34</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="152400" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="40" name="Image 40" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId40"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>9</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="209550" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="41" name="Image 41" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId41"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>12</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="209550" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="42" name="Image 42" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId42"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>15</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="209550" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="43" name="Image 43" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId43"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>18</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="209550" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="44" name="Image 44" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId44"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>21</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="209550" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="45" name="Image 45" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId45"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>24</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="209550" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="46" name="Image 46" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId46"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>27</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="209550" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="47" name="Image 47" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId47"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>30</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="209550" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="48" name="Image 48" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId48"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>33</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="209550" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="49" name="Image 49" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId49"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>36</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="209550" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="50" name="Image 50" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId50"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>39</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="209550" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="51" name="Image 51" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId51"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>42</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="209550" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="52" name="Image 52" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId52"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>45</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="209550" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="53" name="Image 53" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId53"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>48</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="209550" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="54" name="Image 54" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId54"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>51</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="209550" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="55" name="Image 55" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId55"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>54</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="209550" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="56" name="Image 56" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId56"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>57</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="209550" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="57" name="Image 57" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId57"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>60</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="209550" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="58" name="Image 58" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId58"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>63</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="209550" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="59" name="Image 59" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId59"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>66</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="209550" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="60" name="Image 60" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId60"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1667,11 +2497,11 @@
     <ext cx="476250" cy="476250"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="28" name="Image 28" descr="Picture"/>
+        <cNvPr id="61" name="Image 61" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId28"/>
+        <a:blip cstate="print" r:embed="rId61"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1684,7 +2514,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>46</col>
+      <col>77</col>
       <colOff>0</colOff>
       <row>6</row>
       <rowOff>0</rowOff>
@@ -1692,11 +2522,11 @@
     <ext cx="476250" cy="476250"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="29" name="Image 29" descr="Picture"/>
+        <cNvPr id="62" name="Image 62" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId29"/>
+        <a:blip cstate="print" r:embed="rId62"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1717,11 +2547,11 @@
     <ext cx="342900" cy="228600"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="30" name="Image 30" descr="Picture"/>
+        <cNvPr id="63" name="Image 63" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId30"/>
+        <a:blip cstate="print" r:embed="rId63"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1742,11 +2572,11 @@
     <ext cx="342900" cy="228600"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="31" name="Image 31" descr="Picture"/>
+        <cNvPr id="64" name="Image 64" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId31"/>
+        <a:blip cstate="print" r:embed="rId64"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1767,11 +2597,11 @@
     <ext cx="342900" cy="228600"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="32" name="Image 32" descr="Picture"/>
+        <cNvPr id="65" name="Image 65" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId32"/>
+        <a:blip cstate="print" r:embed="rId65"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1792,11 +2622,11 @@
     <ext cx="342900" cy="228600"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="33" name="Image 33" descr="Picture"/>
+        <cNvPr id="66" name="Image 66" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId33"/>
+        <a:blip cstate="print" r:embed="rId66"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1817,11 +2647,11 @@
     <ext cx="342900" cy="228600"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="34" name="Image 34" descr="Picture"/>
+        <cNvPr id="67" name="Image 67" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId34"/>
+        <a:blip cstate="print" r:embed="rId67"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1842,11 +2672,11 @@
     <ext cx="342900" cy="228600"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="35" name="Image 35" descr="Picture"/>
+        <cNvPr id="68" name="Image 68" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId35"/>
+        <a:blip cstate="print" r:embed="rId68"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1867,11 +2697,11 @@
     <ext cx="342900" cy="228600"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="36" name="Image 36" descr="Picture"/>
+        <cNvPr id="69" name="Image 69" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId36"/>
+        <a:blip cstate="print" r:embed="rId69"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -3637,59 +4467,90 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY53"/>
+  <dimension ref="A1:CD53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="2.2" customWidth="1" min="2" max="2"/>
-    <col width="2.2" customWidth="1" min="3" max="3"/>
-    <col width="2.2" customWidth="1" min="4" max="4"/>
-    <col width="2.2" customWidth="1" min="5" max="5"/>
-    <col width="2.2" customWidth="1" min="6" max="6"/>
-    <col width="2.2" customWidth="1" min="7" max="7"/>
-    <col width="2.2" customWidth="1" min="8" max="8"/>
-    <col width="2.2" customWidth="1" min="9" max="9"/>
-    <col width="2.2" customWidth="1" min="10" max="10"/>
-    <col width="2.2" customWidth="1" min="11" max="11"/>
-    <col width="2.2" customWidth="1" min="12" max="12"/>
-    <col width="2.2" customWidth="1" min="13" max="13"/>
-    <col width="2.2" customWidth="1" min="14" max="14"/>
-    <col width="2.2" customWidth="1" min="15" max="15"/>
-    <col width="2.2" customWidth="1" min="16" max="16"/>
-    <col width="2.2" customWidth="1" min="17" max="17"/>
-    <col width="2.2" customWidth="1" min="18" max="18"/>
-    <col width="2.2" customWidth="1" min="19" max="19"/>
-    <col width="2.2" customWidth="1" min="20" max="20"/>
-    <col width="2.2" customWidth="1" min="21" max="21"/>
-    <col width="2.2" customWidth="1" min="22" max="22"/>
-    <col width="2.2" customWidth="1" min="23" max="23"/>
-    <col width="2.2" customWidth="1" min="24" max="24"/>
-    <col width="2.2" customWidth="1" min="25" max="25"/>
-    <col width="2.2" customWidth="1" min="26" max="26"/>
-    <col width="2.2" customWidth="1" min="27" max="27"/>
-    <col width="2.2" customWidth="1" min="28" max="28"/>
-    <col width="2.2" customWidth="1" min="29" max="29"/>
-    <col width="2.2" customWidth="1" min="30" max="30"/>
-    <col width="2.2" customWidth="1" min="31" max="31"/>
-    <col width="2.2" customWidth="1" min="32" max="32"/>
-    <col width="2.2" customWidth="1" min="33" max="33"/>
-    <col width="2.2" customWidth="1" min="34" max="34"/>
-    <col width="2.2" customWidth="1" min="35" max="35"/>
-    <col width="2.2" customWidth="1" min="36" max="36"/>
-    <col width="2.2" customWidth="1" min="37" max="37"/>
-    <col width="2.2" customWidth="1" min="38" max="38"/>
-    <col width="2.2" customWidth="1" min="39" max="39"/>
-    <col width="2.2" customWidth="1" min="40" max="40"/>
-    <col width="2.2" customWidth="1" min="41" max="41"/>
-    <col width="2.2" customWidth="1" min="42" max="42"/>
-    <col width="2.2" customWidth="1" min="43" max="43"/>
-    <col width="2.2" customWidth="1" min="44" max="44"/>
-    <col width="2.2" customWidth="1" min="45" max="45"/>
-    <col width="2.2" customWidth="1" min="46" max="46"/>
-    <col width="2.2" customWidth="1" min="47" max="47"/>
-    <col width="2.2" customWidth="1" min="48" max="48"/>
-    <col width="2.2" customWidth="1" min="49" max="49"/>
-    <col width="2.2" customWidth="1" min="50" max="50"/>
-    <col width="2.2" customWidth="1" min="51" max="51"/>
+    <col width="1.4" customWidth="1" min="2" max="2"/>
+    <col width="1.4" customWidth="1" min="3" max="3"/>
+    <col width="1.4" customWidth="1" min="4" max="4"/>
+    <col width="1.4" customWidth="1" min="5" max="5"/>
+    <col width="1.4" customWidth="1" min="6" max="6"/>
+    <col width="1.4" customWidth="1" min="7" max="7"/>
+    <col width="1.4" customWidth="1" min="8" max="8"/>
+    <col width="1.4" customWidth="1" min="9" max="9"/>
+    <col width="1.4" customWidth="1" min="10" max="10"/>
+    <col width="1.4" customWidth="1" min="11" max="11"/>
+    <col width="1.4" customWidth="1" min="12" max="12"/>
+    <col width="1.4" customWidth="1" min="13" max="13"/>
+    <col width="1.4" customWidth="1" min="14" max="14"/>
+    <col width="1.4" customWidth="1" min="15" max="15"/>
+    <col width="1.4" customWidth="1" min="16" max="16"/>
+    <col width="1.4" customWidth="1" min="17" max="17"/>
+    <col width="1.4" customWidth="1" min="18" max="18"/>
+    <col width="1.4" customWidth="1" min="19" max="19"/>
+    <col width="1.4" customWidth="1" min="20" max="20"/>
+    <col width="1.4" customWidth="1" min="21" max="21"/>
+    <col width="1.4" customWidth="1" min="22" max="22"/>
+    <col width="1.4" customWidth="1" min="23" max="23"/>
+    <col width="1.4" customWidth="1" min="24" max="24"/>
+    <col width="1.4" customWidth="1" min="25" max="25"/>
+    <col width="1.4" customWidth="1" min="26" max="26"/>
+    <col width="1.4" customWidth="1" min="27" max="27"/>
+    <col width="1.4" customWidth="1" min="28" max="28"/>
+    <col width="1.4" customWidth="1" min="29" max="29"/>
+    <col width="1.4" customWidth="1" min="30" max="30"/>
+    <col width="1.4" customWidth="1" min="31" max="31"/>
+    <col width="1.4" customWidth="1" min="32" max="32"/>
+    <col width="1.4" customWidth="1" min="33" max="33"/>
+    <col width="1.4" customWidth="1" min="34" max="34"/>
+    <col width="1.4" customWidth="1" min="35" max="35"/>
+    <col width="1.4" customWidth="1" min="36" max="36"/>
+    <col width="1.4" customWidth="1" min="37" max="37"/>
+    <col width="1.4" customWidth="1" min="38" max="38"/>
+    <col width="1.4" customWidth="1" min="39" max="39"/>
+    <col width="1.4" customWidth="1" min="40" max="40"/>
+    <col width="1.4" customWidth="1" min="41" max="41"/>
+    <col width="1.4" customWidth="1" min="42" max="42"/>
+    <col width="1.4" customWidth="1" min="43" max="43"/>
+    <col width="1.4" customWidth="1" min="44" max="44"/>
+    <col width="1.4" customWidth="1" min="45" max="45"/>
+    <col width="1.4" customWidth="1" min="46" max="46"/>
+    <col width="1.4" customWidth="1" min="47" max="47"/>
+    <col width="1.4" customWidth="1" min="48" max="48"/>
+    <col width="1.4" customWidth="1" min="49" max="49"/>
+    <col width="1.4" customWidth="1" min="50" max="50"/>
+    <col width="1.4" customWidth="1" min="51" max="51"/>
+    <col width="1.4" customWidth="1" min="52" max="52"/>
+    <col width="1.4" customWidth="1" min="53" max="53"/>
+    <col width="1.4" customWidth="1" min="54" max="54"/>
+    <col width="1.4" customWidth="1" min="55" max="55"/>
+    <col width="1.4" customWidth="1" min="56" max="56"/>
+    <col width="1.4" customWidth="1" min="57" max="57"/>
+    <col width="1.4" customWidth="1" min="58" max="58"/>
+    <col width="1.4" customWidth="1" min="59" max="59"/>
+    <col width="1.4" customWidth="1" min="60" max="60"/>
+    <col width="1.4" customWidth="1" min="61" max="61"/>
+    <col width="1.4" customWidth="1" min="62" max="62"/>
+    <col width="1.4" customWidth="1" min="63" max="63"/>
+    <col width="1.4" customWidth="1" min="64" max="64"/>
+    <col width="1.4" customWidth="1" min="65" max="65"/>
+    <col width="1.4" customWidth="1" min="66" max="66"/>
+    <col width="1.4" customWidth="1" min="67" max="67"/>
+    <col width="1.4" customWidth="1" min="68" max="68"/>
+    <col width="1.4" customWidth="1" min="69" max="69"/>
+    <col width="1.4" customWidth="1" min="70" max="70"/>
+    <col width="1.4" customWidth="1" min="71" max="71"/>
+    <col width="1.4" customWidth="1" min="72" max="72"/>
+    <col width="1.4" customWidth="1" min="73" max="73"/>
+    <col width="1.4" customWidth="1" min="74" max="74"/>
+    <col width="1.4" customWidth="1" min="75" max="75"/>
+    <col width="1.4" customWidth="1" min="76" max="76"/>
+    <col width="1.4" customWidth="1" min="77" max="77"/>
+    <col width="1.4" customWidth="1" min="78" max="78"/>
+    <col width="1.4" customWidth="1" min="79" max="79"/>
+    <col width="1.4" customWidth="1" min="80" max="80"/>
+    <col width="1.4" customWidth="1" min="81" max="81"/>
+    <col width="1.4" customWidth="1" min="82" max="82"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -3733,7 +4594,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1 kare = 0.5 m  |  Plan boyutu (varsayilan): 25 m x 18 m</t>
+          <t>1 kare = 0.5 m  |  Plan boyutu (varsayilan): 40 m x 18 m</t>
         </is>
       </c>
     </row>
@@ -3787,7 +4648,38 @@
       <c r="AV7" s="42" t="n"/>
       <c r="AW7" s="42" t="n"/>
       <c r="AX7" s="42" t="n"/>
-      <c r="AY7" s="43" t="n"/>
+      <c r="AY7" s="42" t="n"/>
+      <c r="AZ7" s="42" t="n"/>
+      <c r="BA7" s="42" t="n"/>
+      <c r="BB7" s="42" t="n"/>
+      <c r="BC7" s="42" t="n"/>
+      <c r="BD7" s="42" t="n"/>
+      <c r="BE7" s="42" t="n"/>
+      <c r="BF7" s="42" t="n"/>
+      <c r="BG7" s="42" t="n"/>
+      <c r="BH7" s="42" t="n"/>
+      <c r="BI7" s="42" t="n"/>
+      <c r="BJ7" s="42" t="n"/>
+      <c r="BK7" s="42" t="n"/>
+      <c r="BL7" s="42" t="n"/>
+      <c r="BM7" s="42" t="n"/>
+      <c r="BN7" s="42" t="n"/>
+      <c r="BO7" s="42" t="n"/>
+      <c r="BP7" s="42" t="n"/>
+      <c r="BQ7" s="42" t="n"/>
+      <c r="BR7" s="42" t="n"/>
+      <c r="BS7" s="42" t="n"/>
+      <c r="BT7" s="42" t="n"/>
+      <c r="BU7" s="42" t="n"/>
+      <c r="BV7" s="42" t="n"/>
+      <c r="BW7" s="42" t="n"/>
+      <c r="BX7" s="42" t="n"/>
+      <c r="BY7" s="42" t="n"/>
+      <c r="BZ7" s="42" t="n"/>
+      <c r="CA7" s="42" t="n"/>
+      <c r="CB7" s="42" t="n"/>
+      <c r="CC7" s="42" t="n"/>
+      <c r="CD7" s="43" t="n"/>
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="B8" s="44" t="n"/>
@@ -3839,7 +4731,38 @@
       <c r="AV8" s="45" t="n"/>
       <c r="AW8" s="45" t="n"/>
       <c r="AX8" s="45" t="n"/>
-      <c r="AY8" s="46" t="n"/>
+      <c r="AY8" s="45" t="n"/>
+      <c r="AZ8" s="45" t="n"/>
+      <c r="BA8" s="45" t="n"/>
+      <c r="BB8" s="45" t="n"/>
+      <c r="BC8" s="45" t="n"/>
+      <c r="BD8" s="45" t="n"/>
+      <c r="BE8" s="45" t="n"/>
+      <c r="BF8" s="45" t="n"/>
+      <c r="BG8" s="45" t="n"/>
+      <c r="BH8" s="45" t="n"/>
+      <c r="BI8" s="45" t="n"/>
+      <c r="BJ8" s="45" t="n"/>
+      <c r="BK8" s="45" t="n"/>
+      <c r="BL8" s="45" t="n"/>
+      <c r="BM8" s="45" t="n"/>
+      <c r="BN8" s="45" t="n"/>
+      <c r="BO8" s="45" t="n"/>
+      <c r="BP8" s="45" t="n"/>
+      <c r="BQ8" s="45" t="n"/>
+      <c r="BR8" s="45" t="n"/>
+      <c r="BS8" s="45" t="n"/>
+      <c r="BT8" s="45" t="n"/>
+      <c r="BU8" s="45" t="n"/>
+      <c r="BV8" s="45" t="n"/>
+      <c r="BW8" s="45" t="n"/>
+      <c r="BX8" s="45" t="n"/>
+      <c r="BY8" s="45" t="n"/>
+      <c r="BZ8" s="45" t="n"/>
+      <c r="CA8" s="45" t="n"/>
+      <c r="CB8" s="45" t="n"/>
+      <c r="CC8" s="45" t="n"/>
+      <c r="CD8" s="46" t="n"/>
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="B9" s="44" t="n"/>
@@ -3891,7 +4814,38 @@
       <c r="AV9" s="45" t="n"/>
       <c r="AW9" s="45" t="n"/>
       <c r="AX9" s="45" t="n"/>
-      <c r="AY9" s="46" t="n"/>
+      <c r="AY9" s="45" t="n"/>
+      <c r="AZ9" s="45" t="n"/>
+      <c r="BA9" s="45" t="n"/>
+      <c r="BB9" s="45" t="n"/>
+      <c r="BC9" s="45" t="n"/>
+      <c r="BD9" s="45" t="n"/>
+      <c r="BE9" s="45" t="n"/>
+      <c r="BF9" s="45" t="n"/>
+      <c r="BG9" s="45" t="n"/>
+      <c r="BH9" s="45" t="n"/>
+      <c r="BI9" s="45" t="n"/>
+      <c r="BJ9" s="45" t="n"/>
+      <c r="BK9" s="45" t="n"/>
+      <c r="BL9" s="45" t="n"/>
+      <c r="BM9" s="45" t="n"/>
+      <c r="BN9" s="45" t="n"/>
+      <c r="BO9" s="45" t="n"/>
+      <c r="BP9" s="45" t="n"/>
+      <c r="BQ9" s="45" t="n"/>
+      <c r="BR9" s="45" t="n"/>
+      <c r="BS9" s="45" t="n"/>
+      <c r="BT9" s="45" t="n"/>
+      <c r="BU9" s="45" t="n"/>
+      <c r="BV9" s="45" t="n"/>
+      <c r="BW9" s="45" t="n"/>
+      <c r="BX9" s="45" t="n"/>
+      <c r="BY9" s="45" t="n"/>
+      <c r="BZ9" s="45" t="n"/>
+      <c r="CA9" s="45" t="n"/>
+      <c r="CB9" s="45" t="n"/>
+      <c r="CC9" s="45" t="n"/>
+      <c r="CD9" s="46" t="n"/>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="B10" s="44" t="n"/>
@@ -3903,47 +4857,78 @@
       <c r="H10" s="47" t="n"/>
       <c r="I10" s="47" t="n"/>
       <c r="J10" s="47" t="n"/>
-      <c r="K10" s="47" t="n"/>
-      <c r="L10" s="48" t="n"/>
+      <c r="K10" s="48" t="n"/>
+      <c r="L10" s="47" t="n"/>
       <c r="M10" s="47" t="n"/>
-      <c r="N10" s="47" t="n"/>
+      <c r="N10" s="48" t="n"/>
       <c r="O10" s="47" t="n"/>
       <c r="P10" s="47" t="n"/>
-      <c r="Q10" s="47" t="n"/>
+      <c r="Q10" s="48" t="n"/>
       <c r="R10" s="47" t="n"/>
       <c r="S10" s="47" t="n"/>
-      <c r="T10" s="47" t="n"/>
+      <c r="T10" s="48" t="n"/>
       <c r="U10" s="47" t="n"/>
       <c r="V10" s="47" t="n"/>
-      <c r="W10" s="47" t="n"/>
-      <c r="X10" s="48" t="n"/>
+      <c r="W10" s="48" t="n"/>
+      <c r="X10" s="47" t="n"/>
       <c r="Y10" s="47" t="n"/>
-      <c r="Z10" s="47" t="n"/>
+      <c r="Z10" s="48" t="n"/>
       <c r="AA10" s="47" t="n"/>
       <c r="AB10" s="47" t="n"/>
-      <c r="AC10" s="47" t="n"/>
+      <c r="AC10" s="48" t="n"/>
       <c r="AD10" s="47" t="n"/>
       <c r="AE10" s="47" t="n"/>
-      <c r="AF10" s="47" t="n"/>
+      <c r="AF10" s="48" t="n"/>
       <c r="AG10" s="47" t="n"/>
       <c r="AH10" s="47" t="n"/>
-      <c r="AI10" s="47" t="n"/>
-      <c r="AJ10" s="48" t="n"/>
+      <c r="AI10" s="48" t="n"/>
+      <c r="AJ10" s="47" t="n"/>
       <c r="AK10" s="47" t="n"/>
-      <c r="AL10" s="47" t="n"/>
+      <c r="AL10" s="48" t="n"/>
       <c r="AM10" s="47" t="n"/>
       <c r="AN10" s="47" t="n"/>
-      <c r="AO10" s="47" t="n"/>
+      <c r="AO10" s="48" t="n"/>
       <c r="AP10" s="47" t="n"/>
       <c r="AQ10" s="47" t="n"/>
-      <c r="AR10" s="47" t="n"/>
+      <c r="AR10" s="48" t="n"/>
       <c r="AS10" s="47" t="n"/>
-      <c r="AT10" s="45" t="n"/>
-      <c r="AU10" s="45" t="n"/>
-      <c r="AV10" s="45" t="n"/>
-      <c r="AW10" s="45" t="n"/>
-      <c r="AX10" s="45" t="n"/>
-      <c r="AY10" s="46" t="n"/>
+      <c r="AT10" s="47" t="n"/>
+      <c r="AU10" s="48" t="n"/>
+      <c r="AV10" s="47" t="n"/>
+      <c r="AW10" s="47" t="n"/>
+      <c r="AX10" s="48" t="n"/>
+      <c r="AY10" s="47" t="n"/>
+      <c r="AZ10" s="47" t="n"/>
+      <c r="BA10" s="48" t="n"/>
+      <c r="BB10" s="47" t="n"/>
+      <c r="BC10" s="47" t="n"/>
+      <c r="BD10" s="48" t="n"/>
+      <c r="BE10" s="47" t="n"/>
+      <c r="BF10" s="47" t="n"/>
+      <c r="BG10" s="48" t="n"/>
+      <c r="BH10" s="47" t="n"/>
+      <c r="BI10" s="47" t="n"/>
+      <c r="BJ10" s="48" t="n"/>
+      <c r="BK10" s="47" t="n"/>
+      <c r="BL10" s="47" t="n"/>
+      <c r="BM10" s="48" t="n"/>
+      <c r="BN10" s="47" t="n"/>
+      <c r="BO10" s="47" t="n"/>
+      <c r="BP10" s="48" t="n"/>
+      <c r="BQ10" s="47" t="n"/>
+      <c r="BR10" s="47" t="n"/>
+      <c r="BS10" s="47" t="n"/>
+      <c r="BT10" s="47" t="n"/>
+      <c r="BU10" s="47" t="n"/>
+      <c r="BV10" s="47" t="n"/>
+      <c r="BW10" s="47" t="n"/>
+      <c r="BX10" s="47" t="n"/>
+      <c r="BY10" s="45" t="n"/>
+      <c r="BZ10" s="45" t="n"/>
+      <c r="CA10" s="45" t="n"/>
+      <c r="CB10" s="45" t="n"/>
+      <c r="CC10" s="45" t="n"/>
+      <c r="CD10" s="46" t="n"/>
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="B11" s="44" t="n"/>
@@ -3958,50 +4943,81 @@
       <c r="H11" s="45" t="n"/>
       <c r="I11" s="45" t="n"/>
       <c r="J11" s="45" t="n"/>
-      <c r="K11" s="45" t="n"/>
-      <c r="L11" s="50" t="n"/>
+      <c r="K11" s="50" t="n"/>
+      <c r="L11" s="45" t="n"/>
       <c r="M11" s="45" t="n"/>
-      <c r="N11" s="45" t="n"/>
+      <c r="N11" s="50" t="n"/>
       <c r="O11" s="45" t="n"/>
       <c r="P11" s="45" t="n"/>
-      <c r="Q11" s="45" t="n"/>
+      <c r="Q11" s="50" t="n"/>
       <c r="R11" s="45" t="n"/>
       <c r="S11" s="45" t="n"/>
-      <c r="T11" s="45" t="n"/>
+      <c r="T11" s="50" t="n"/>
       <c r="U11" s="45" t="n"/>
       <c r="V11" s="45" t="n"/>
-      <c r="W11" s="45" t="n"/>
-      <c r="X11" s="50" t="n"/>
+      <c r="W11" s="50" t="n"/>
+      <c r="X11" s="45" t="n"/>
       <c r="Y11" s="45" t="n"/>
-      <c r="Z11" s="45" t="n"/>
+      <c r="Z11" s="50" t="n"/>
       <c r="AA11" s="45" t="n"/>
       <c r="AB11" s="45" t="n"/>
-      <c r="AC11" s="45" t="n"/>
+      <c r="AC11" s="50" t="n"/>
       <c r="AD11" s="45" t="n"/>
       <c r="AE11" s="45" t="n"/>
-      <c r="AF11" s="45" t="n"/>
+      <c r="AF11" s="50" t="n"/>
       <c r="AG11" s="45" t="n"/>
       <c r="AH11" s="45" t="n"/>
-      <c r="AI11" s="45" t="n"/>
-      <c r="AJ11" s="50" t="n"/>
+      <c r="AI11" s="50" t="n"/>
+      <c r="AJ11" s="45" t="n"/>
       <c r="AK11" s="45" t="n"/>
-      <c r="AL11" s="45" t="n"/>
+      <c r="AL11" s="50" t="n"/>
       <c r="AM11" s="45" t="n"/>
       <c r="AN11" s="45" t="n"/>
-      <c r="AO11" s="45" t="n"/>
+      <c r="AO11" s="50" t="n"/>
       <c r="AP11" s="45" t="n"/>
       <c r="AQ11" s="45" t="n"/>
-      <c r="AR11" s="45" t="n"/>
+      <c r="AR11" s="50" t="n"/>
       <c r="AS11" s="45" t="n"/>
       <c r="AT11" s="45" t="n"/>
-      <c r="AU11" s="49">
+      <c r="AU11" s="50" t="n"/>
+      <c r="AV11" s="45" t="n"/>
+      <c r="AW11" s="45" t="n"/>
+      <c r="AX11" s="50" t="n"/>
+      <c r="AY11" s="45" t="n"/>
+      <c r="AZ11" s="45" t="n"/>
+      <c r="BA11" s="50" t="n"/>
+      <c r="BB11" s="45" t="n"/>
+      <c r="BC11" s="45" t="n"/>
+      <c r="BD11" s="50" t="n"/>
+      <c r="BE11" s="45" t="n"/>
+      <c r="BF11" s="45" t="n"/>
+      <c r="BG11" s="50" t="n"/>
+      <c r="BH11" s="45" t="n"/>
+      <c r="BI11" s="45" t="n"/>
+      <c r="BJ11" s="50" t="n"/>
+      <c r="BK11" s="45" t="n"/>
+      <c r="BL11" s="45" t="n"/>
+      <c r="BM11" s="50" t="n"/>
+      <c r="BN11" s="45" t="n"/>
+      <c r="BO11" s="45" t="n"/>
+      <c r="BP11" s="50" t="n"/>
+      <c r="BQ11" s="45" t="n"/>
+      <c r="BR11" s="45" t="n"/>
+      <c r="BS11" s="45" t="n"/>
+      <c r="BT11" s="45" t="n"/>
+      <c r="BU11" s="45" t="n"/>
+      <c r="BV11" s="45" t="n"/>
+      <c r="BW11" s="45" t="n"/>
+      <c r="BX11" s="45" t="n"/>
+      <c r="BY11" s="45" t="n"/>
+      <c r="BZ11" s="49">
         <f>'Fan Secimi'!B14</f>
         <v/>
       </c>
-      <c r="AV11" s="51" t="n"/>
-      <c r="AW11" s="51" t="n"/>
-      <c r="AX11" s="52" t="n"/>
-      <c r="AY11" s="46" t="n"/>
+      <c r="CA11" s="51" t="n"/>
+      <c r="CB11" s="51" t="n"/>
+      <c r="CC11" s="52" t="n"/>
+      <c r="CD11" s="46" t="n"/>
     </row>
     <row r="12" ht="15" customHeight="1">
       <c r="B12" s="44" t="n"/>
@@ -4013,47 +5029,78 @@
       <c r="H12" s="45" t="n"/>
       <c r="I12" s="45" t="n"/>
       <c r="J12" s="45" t="n"/>
-      <c r="K12" s="45" t="n"/>
-      <c r="L12" s="50" t="n"/>
+      <c r="K12" s="50" t="n"/>
+      <c r="L12" s="45" t="n"/>
       <c r="M12" s="45" t="n"/>
-      <c r="N12" s="45" t="n"/>
+      <c r="N12" s="50" t="n"/>
       <c r="O12" s="45" t="n"/>
       <c r="P12" s="45" t="n"/>
-      <c r="Q12" s="45" t="n"/>
+      <c r="Q12" s="50" t="n"/>
       <c r="R12" s="45" t="n"/>
       <c r="S12" s="45" t="n"/>
-      <c r="T12" s="45" t="n"/>
+      <c r="T12" s="50" t="n"/>
       <c r="U12" s="45" t="n"/>
       <c r="V12" s="45" t="n"/>
-      <c r="W12" s="45" t="n"/>
-      <c r="X12" s="50" t="n"/>
+      <c r="W12" s="50" t="n"/>
+      <c r="X12" s="45" t="n"/>
       <c r="Y12" s="45" t="n"/>
-      <c r="Z12" s="45" t="n"/>
+      <c r="Z12" s="50" t="n"/>
       <c r="AA12" s="45" t="n"/>
       <c r="AB12" s="45" t="n"/>
-      <c r="AC12" s="45" t="n"/>
+      <c r="AC12" s="50" t="n"/>
       <c r="AD12" s="45" t="n"/>
       <c r="AE12" s="45" t="n"/>
-      <c r="AF12" s="45" t="n"/>
+      <c r="AF12" s="50" t="n"/>
       <c r="AG12" s="45" t="n"/>
       <c r="AH12" s="45" t="n"/>
-      <c r="AI12" s="45" t="n"/>
-      <c r="AJ12" s="50" t="n"/>
+      <c r="AI12" s="50" t="n"/>
+      <c r="AJ12" s="45" t="n"/>
       <c r="AK12" s="45" t="n"/>
-      <c r="AL12" s="45" t="n"/>
+      <c r="AL12" s="50" t="n"/>
       <c r="AM12" s="45" t="n"/>
       <c r="AN12" s="45" t="n"/>
-      <c r="AO12" s="45" t="n"/>
+      <c r="AO12" s="50" t="n"/>
       <c r="AP12" s="45" t="n"/>
       <c r="AQ12" s="45" t="n"/>
-      <c r="AR12" s="45" t="n"/>
+      <c r="AR12" s="50" t="n"/>
       <c r="AS12" s="45" t="n"/>
       <c r="AT12" s="45" t="n"/>
-      <c r="AU12" s="45" t="n"/>
+      <c r="AU12" s="50" t="n"/>
       <c r="AV12" s="45" t="n"/>
       <c r="AW12" s="45" t="n"/>
-      <c r="AX12" s="45" t="n"/>
-      <c r="AY12" s="46" t="n"/>
+      <c r="AX12" s="50" t="n"/>
+      <c r="AY12" s="45" t="n"/>
+      <c r="AZ12" s="45" t="n"/>
+      <c r="BA12" s="50" t="n"/>
+      <c r="BB12" s="45" t="n"/>
+      <c r="BC12" s="45" t="n"/>
+      <c r="BD12" s="50" t="n"/>
+      <c r="BE12" s="45" t="n"/>
+      <c r="BF12" s="45" t="n"/>
+      <c r="BG12" s="50" t="n"/>
+      <c r="BH12" s="45" t="n"/>
+      <c r="BI12" s="45" t="n"/>
+      <c r="BJ12" s="50" t="n"/>
+      <c r="BK12" s="45" t="n"/>
+      <c r="BL12" s="45" t="n"/>
+      <c r="BM12" s="50" t="n"/>
+      <c r="BN12" s="45" t="n"/>
+      <c r="BO12" s="45" t="n"/>
+      <c r="BP12" s="50" t="n"/>
+      <c r="BQ12" s="45" t="n"/>
+      <c r="BR12" s="45" t="n"/>
+      <c r="BS12" s="45" t="n"/>
+      <c r="BT12" s="45" t="n"/>
+      <c r="BU12" s="45" t="n"/>
+      <c r="BV12" s="45" t="n"/>
+      <c r="BW12" s="45" t="n"/>
+      <c r="BX12" s="45" t="n"/>
+      <c r="BY12" s="45" t="n"/>
+      <c r="BZ12" s="45" t="n"/>
+      <c r="CA12" s="45" t="n"/>
+      <c r="CB12" s="45" t="n"/>
+      <c r="CC12" s="45" t="n"/>
+      <c r="CD12" s="46" t="n"/>
     </row>
     <row r="13" ht="15" customHeight="1">
       <c r="B13" s="44" t="n"/>
@@ -4065,47 +5112,78 @@
       <c r="H13" s="45" t="n"/>
       <c r="I13" s="45" t="n"/>
       <c r="J13" s="45" t="n"/>
-      <c r="K13" s="45" t="n"/>
-      <c r="L13" s="50" t="n"/>
+      <c r="K13" s="50" t="n"/>
+      <c r="L13" s="45" t="n"/>
       <c r="M13" s="45" t="n"/>
-      <c r="N13" s="45" t="n"/>
+      <c r="N13" s="50" t="n"/>
       <c r="O13" s="45" t="n"/>
       <c r="P13" s="45" t="n"/>
-      <c r="Q13" s="45" t="n"/>
+      <c r="Q13" s="50" t="n"/>
       <c r="R13" s="45" t="n"/>
       <c r="S13" s="45" t="n"/>
-      <c r="T13" s="45" t="n"/>
+      <c r="T13" s="50" t="n"/>
       <c r="U13" s="45" t="n"/>
       <c r="V13" s="45" t="n"/>
-      <c r="W13" s="45" t="n"/>
-      <c r="X13" s="50" t="n"/>
+      <c r="W13" s="50" t="n"/>
+      <c r="X13" s="45" t="n"/>
       <c r="Y13" s="45" t="n"/>
-      <c r="Z13" s="45" t="n"/>
+      <c r="Z13" s="50" t="n"/>
       <c r="AA13" s="45" t="n"/>
       <c r="AB13" s="45" t="n"/>
-      <c r="AC13" s="45" t="n"/>
+      <c r="AC13" s="50" t="n"/>
       <c r="AD13" s="45" t="n"/>
       <c r="AE13" s="45" t="n"/>
-      <c r="AF13" s="45" t="n"/>
+      <c r="AF13" s="50" t="n"/>
       <c r="AG13" s="45" t="n"/>
       <c r="AH13" s="45" t="n"/>
-      <c r="AI13" s="45" t="n"/>
-      <c r="AJ13" s="50" t="n"/>
+      <c r="AI13" s="50" t="n"/>
+      <c r="AJ13" s="45" t="n"/>
       <c r="AK13" s="45" t="n"/>
-      <c r="AL13" s="45" t="n"/>
+      <c r="AL13" s="50" t="n"/>
       <c r="AM13" s="45" t="n"/>
       <c r="AN13" s="45" t="n"/>
-      <c r="AO13" s="45" t="n"/>
+      <c r="AO13" s="50" t="n"/>
       <c r="AP13" s="45" t="n"/>
       <c r="AQ13" s="45" t="n"/>
-      <c r="AR13" s="45" t="n"/>
+      <c r="AR13" s="50" t="n"/>
       <c r="AS13" s="45" t="n"/>
       <c r="AT13" s="45" t="n"/>
-      <c r="AU13" s="45" t="n"/>
+      <c r="AU13" s="50" t="n"/>
       <c r="AV13" s="45" t="n"/>
       <c r="AW13" s="45" t="n"/>
-      <c r="AX13" s="45" t="n"/>
-      <c r="AY13" s="46" t="n"/>
+      <c r="AX13" s="50" t="n"/>
+      <c r="AY13" s="45" t="n"/>
+      <c r="AZ13" s="45" t="n"/>
+      <c r="BA13" s="50" t="n"/>
+      <c r="BB13" s="45" t="n"/>
+      <c r="BC13" s="45" t="n"/>
+      <c r="BD13" s="50" t="n"/>
+      <c r="BE13" s="45" t="n"/>
+      <c r="BF13" s="45" t="n"/>
+      <c r="BG13" s="50" t="n"/>
+      <c r="BH13" s="45" t="n"/>
+      <c r="BI13" s="45" t="n"/>
+      <c r="BJ13" s="50" t="n"/>
+      <c r="BK13" s="45" t="n"/>
+      <c r="BL13" s="45" t="n"/>
+      <c r="BM13" s="50" t="n"/>
+      <c r="BN13" s="45" t="n"/>
+      <c r="BO13" s="45" t="n"/>
+      <c r="BP13" s="50" t="n"/>
+      <c r="BQ13" s="45" t="n"/>
+      <c r="BR13" s="45" t="n"/>
+      <c r="BS13" s="45" t="n"/>
+      <c r="BT13" s="45" t="n"/>
+      <c r="BU13" s="45" t="n"/>
+      <c r="BV13" s="45" t="n"/>
+      <c r="BW13" s="45" t="n"/>
+      <c r="BX13" s="45" t="n"/>
+      <c r="BY13" s="45" t="n"/>
+      <c r="BZ13" s="45" t="n"/>
+      <c r="CA13" s="45" t="n"/>
+      <c r="CB13" s="45" t="n"/>
+      <c r="CC13" s="45" t="n"/>
+      <c r="CD13" s="46" t="n"/>
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="B14" s="44" t="n"/>
@@ -4117,47 +5195,78 @@
       <c r="H14" s="45" t="n"/>
       <c r="I14" s="45" t="n"/>
       <c r="J14" s="45" t="n"/>
-      <c r="K14" s="45" t="n"/>
-      <c r="L14" s="50" t="n"/>
+      <c r="K14" s="50" t="n"/>
+      <c r="L14" s="45" t="n"/>
       <c r="M14" s="45" t="n"/>
-      <c r="N14" s="45" t="n"/>
+      <c r="N14" s="50" t="n"/>
       <c r="O14" s="45" t="n"/>
       <c r="P14" s="45" t="n"/>
-      <c r="Q14" s="45" t="n"/>
+      <c r="Q14" s="50" t="n"/>
       <c r="R14" s="45" t="n"/>
       <c r="S14" s="45" t="n"/>
-      <c r="T14" s="45" t="n"/>
+      <c r="T14" s="50" t="n"/>
       <c r="U14" s="45" t="n"/>
       <c r="V14" s="45" t="n"/>
-      <c r="W14" s="45" t="n"/>
-      <c r="X14" s="50" t="n"/>
+      <c r="W14" s="50" t="n"/>
+      <c r="X14" s="45" t="n"/>
       <c r="Y14" s="45" t="n"/>
-      <c r="Z14" s="45" t="n"/>
+      <c r="Z14" s="50" t="n"/>
       <c r="AA14" s="45" t="n"/>
       <c r="AB14" s="45" t="n"/>
-      <c r="AC14" s="45" t="n"/>
+      <c r="AC14" s="50" t="n"/>
       <c r="AD14" s="45" t="n"/>
       <c r="AE14" s="45" t="n"/>
-      <c r="AF14" s="45" t="n"/>
+      <c r="AF14" s="50" t="n"/>
       <c r="AG14" s="45" t="n"/>
       <c r="AH14" s="45" t="n"/>
-      <c r="AI14" s="45" t="n"/>
-      <c r="AJ14" s="50" t="n"/>
+      <c r="AI14" s="50" t="n"/>
+      <c r="AJ14" s="45" t="n"/>
       <c r="AK14" s="45" t="n"/>
-      <c r="AL14" s="45" t="n"/>
+      <c r="AL14" s="50" t="n"/>
       <c r="AM14" s="45" t="n"/>
       <c r="AN14" s="45" t="n"/>
-      <c r="AO14" s="45" t="n"/>
+      <c r="AO14" s="50" t="n"/>
       <c r="AP14" s="45" t="n"/>
       <c r="AQ14" s="45" t="n"/>
-      <c r="AR14" s="45" t="n"/>
+      <c r="AR14" s="50" t="n"/>
       <c r="AS14" s="45" t="n"/>
       <c r="AT14" s="45" t="n"/>
-      <c r="AU14" s="45" t="n"/>
+      <c r="AU14" s="50" t="n"/>
       <c r="AV14" s="45" t="n"/>
       <c r="AW14" s="45" t="n"/>
-      <c r="AX14" s="45" t="n"/>
-      <c r="AY14" s="46" t="n"/>
+      <c r="AX14" s="50" t="n"/>
+      <c r="AY14" s="45" t="n"/>
+      <c r="AZ14" s="45" t="n"/>
+      <c r="BA14" s="50" t="n"/>
+      <c r="BB14" s="45" t="n"/>
+      <c r="BC14" s="45" t="n"/>
+      <c r="BD14" s="50" t="n"/>
+      <c r="BE14" s="45" t="n"/>
+      <c r="BF14" s="45" t="n"/>
+      <c r="BG14" s="50" t="n"/>
+      <c r="BH14" s="45" t="n"/>
+      <c r="BI14" s="45" t="n"/>
+      <c r="BJ14" s="50" t="n"/>
+      <c r="BK14" s="45" t="n"/>
+      <c r="BL14" s="45" t="n"/>
+      <c r="BM14" s="50" t="n"/>
+      <c r="BN14" s="45" t="n"/>
+      <c r="BO14" s="45" t="n"/>
+      <c r="BP14" s="50" t="n"/>
+      <c r="BQ14" s="45" t="n"/>
+      <c r="BR14" s="45" t="n"/>
+      <c r="BS14" s="45" t="n"/>
+      <c r="BT14" s="45" t="n"/>
+      <c r="BU14" s="45" t="n"/>
+      <c r="BV14" s="45" t="n"/>
+      <c r="BW14" s="45" t="n"/>
+      <c r="BX14" s="45" t="n"/>
+      <c r="BY14" s="45" t="n"/>
+      <c r="BZ14" s="45" t="n"/>
+      <c r="CA14" s="45" t="n"/>
+      <c r="CB14" s="45" t="n"/>
+      <c r="CC14" s="45" t="n"/>
+      <c r="CD14" s="46" t="n"/>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="B15" s="44" t="n"/>
@@ -4169,47 +5278,78 @@
       <c r="H15" s="45" t="n"/>
       <c r="I15" s="45" t="n"/>
       <c r="J15" s="45" t="n"/>
-      <c r="K15" s="45" t="n"/>
-      <c r="L15" s="50" t="n"/>
+      <c r="K15" s="50" t="n"/>
+      <c r="L15" s="45" t="n"/>
       <c r="M15" s="45" t="n"/>
-      <c r="N15" s="45" t="n"/>
+      <c r="N15" s="50" t="n"/>
       <c r="O15" s="45" t="n"/>
       <c r="P15" s="45" t="n"/>
-      <c r="Q15" s="45" t="n"/>
+      <c r="Q15" s="50" t="n"/>
       <c r="R15" s="45" t="n"/>
       <c r="S15" s="45" t="n"/>
-      <c r="T15" s="45" t="n"/>
+      <c r="T15" s="50" t="n"/>
       <c r="U15" s="45" t="n"/>
       <c r="V15" s="45" t="n"/>
-      <c r="W15" s="45" t="n"/>
-      <c r="X15" s="50" t="n"/>
+      <c r="W15" s="50" t="n"/>
+      <c r="X15" s="45" t="n"/>
       <c r="Y15" s="45" t="n"/>
-      <c r="Z15" s="45" t="n"/>
+      <c r="Z15" s="50" t="n"/>
       <c r="AA15" s="45" t="n"/>
       <c r="AB15" s="45" t="n"/>
-      <c r="AC15" s="45" t="n"/>
+      <c r="AC15" s="50" t="n"/>
       <c r="AD15" s="45" t="n"/>
       <c r="AE15" s="45" t="n"/>
-      <c r="AF15" s="45" t="n"/>
+      <c r="AF15" s="50" t="n"/>
       <c r="AG15" s="45" t="n"/>
       <c r="AH15" s="45" t="n"/>
-      <c r="AI15" s="45" t="n"/>
-      <c r="AJ15" s="50" t="n"/>
+      <c r="AI15" s="50" t="n"/>
+      <c r="AJ15" s="45" t="n"/>
       <c r="AK15" s="45" t="n"/>
-      <c r="AL15" s="45" t="n"/>
+      <c r="AL15" s="50" t="n"/>
       <c r="AM15" s="45" t="n"/>
       <c r="AN15" s="45" t="n"/>
-      <c r="AO15" s="45" t="n"/>
+      <c r="AO15" s="50" t="n"/>
       <c r="AP15" s="45" t="n"/>
       <c r="AQ15" s="45" t="n"/>
-      <c r="AR15" s="45" t="n"/>
+      <c r="AR15" s="50" t="n"/>
       <c r="AS15" s="45" t="n"/>
       <c r="AT15" s="45" t="n"/>
-      <c r="AU15" s="45" t="n"/>
+      <c r="AU15" s="50" t="n"/>
       <c r="AV15" s="45" t="n"/>
       <c r="AW15" s="45" t="n"/>
-      <c r="AX15" s="45" t="n"/>
-      <c r="AY15" s="46" t="n"/>
+      <c r="AX15" s="50" t="n"/>
+      <c r="AY15" s="45" t="n"/>
+      <c r="AZ15" s="45" t="n"/>
+      <c r="BA15" s="50" t="n"/>
+      <c r="BB15" s="45" t="n"/>
+      <c r="BC15" s="45" t="n"/>
+      <c r="BD15" s="50" t="n"/>
+      <c r="BE15" s="45" t="n"/>
+      <c r="BF15" s="45" t="n"/>
+      <c r="BG15" s="50" t="n"/>
+      <c r="BH15" s="45" t="n"/>
+      <c r="BI15" s="45" t="n"/>
+      <c r="BJ15" s="50" t="n"/>
+      <c r="BK15" s="45" t="n"/>
+      <c r="BL15" s="45" t="n"/>
+      <c r="BM15" s="50" t="n"/>
+      <c r="BN15" s="45" t="n"/>
+      <c r="BO15" s="45" t="n"/>
+      <c r="BP15" s="50" t="n"/>
+      <c r="BQ15" s="45" t="n"/>
+      <c r="BR15" s="45" t="n"/>
+      <c r="BS15" s="45" t="n"/>
+      <c r="BT15" s="45" t="n"/>
+      <c r="BU15" s="45" t="n"/>
+      <c r="BV15" s="45" t="n"/>
+      <c r="BW15" s="45" t="n"/>
+      <c r="BX15" s="45" t="n"/>
+      <c r="BY15" s="45" t="n"/>
+      <c r="BZ15" s="45" t="n"/>
+      <c r="CA15" s="45" t="n"/>
+      <c r="CB15" s="45" t="n"/>
+      <c r="CC15" s="45" t="n"/>
+      <c r="CD15" s="46" t="n"/>
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="B16" s="44" t="n"/>
@@ -4221,47 +5361,78 @@
       <c r="H16" s="45" t="n"/>
       <c r="I16" s="45" t="n"/>
       <c r="J16" s="45" t="n"/>
-      <c r="K16" s="45" t="n"/>
-      <c r="L16" s="50" t="n"/>
+      <c r="K16" s="50" t="n"/>
+      <c r="L16" s="45" t="n"/>
       <c r="M16" s="45" t="n"/>
-      <c r="N16" s="45" t="n"/>
+      <c r="N16" s="50" t="n"/>
       <c r="O16" s="45" t="n"/>
       <c r="P16" s="45" t="n"/>
-      <c r="Q16" s="45" t="n"/>
+      <c r="Q16" s="50" t="n"/>
       <c r="R16" s="45" t="n"/>
       <c r="S16" s="45" t="n"/>
-      <c r="T16" s="45" t="n"/>
+      <c r="T16" s="50" t="n"/>
       <c r="U16" s="45" t="n"/>
       <c r="V16" s="45" t="n"/>
-      <c r="W16" s="45" t="n"/>
-      <c r="X16" s="50" t="n"/>
+      <c r="W16" s="50" t="n"/>
+      <c r="X16" s="45" t="n"/>
       <c r="Y16" s="45" t="n"/>
-      <c r="Z16" s="45" t="n"/>
+      <c r="Z16" s="50" t="n"/>
       <c r="AA16" s="45" t="n"/>
       <c r="AB16" s="45" t="n"/>
-      <c r="AC16" s="45" t="n"/>
+      <c r="AC16" s="50" t="n"/>
       <c r="AD16" s="45" t="n"/>
       <c r="AE16" s="45" t="n"/>
-      <c r="AF16" s="45" t="n"/>
+      <c r="AF16" s="50" t="n"/>
       <c r="AG16" s="45" t="n"/>
       <c r="AH16" s="45" t="n"/>
-      <c r="AI16" s="45" t="n"/>
-      <c r="AJ16" s="50" t="n"/>
+      <c r="AI16" s="50" t="n"/>
+      <c r="AJ16" s="45" t="n"/>
       <c r="AK16" s="45" t="n"/>
-      <c r="AL16" s="45" t="n"/>
+      <c r="AL16" s="50" t="n"/>
       <c r="AM16" s="45" t="n"/>
       <c r="AN16" s="45" t="n"/>
-      <c r="AO16" s="45" t="n"/>
+      <c r="AO16" s="50" t="n"/>
       <c r="AP16" s="45" t="n"/>
       <c r="AQ16" s="45" t="n"/>
-      <c r="AR16" s="45" t="n"/>
+      <c r="AR16" s="50" t="n"/>
       <c r="AS16" s="45" t="n"/>
       <c r="AT16" s="45" t="n"/>
-      <c r="AU16" s="45" t="n"/>
+      <c r="AU16" s="50" t="n"/>
       <c r="AV16" s="45" t="n"/>
       <c r="AW16" s="45" t="n"/>
-      <c r="AX16" s="45" t="n"/>
-      <c r="AY16" s="46" t="n"/>
+      <c r="AX16" s="50" t="n"/>
+      <c r="AY16" s="45" t="n"/>
+      <c r="AZ16" s="45" t="n"/>
+      <c r="BA16" s="50" t="n"/>
+      <c r="BB16" s="45" t="n"/>
+      <c r="BC16" s="45" t="n"/>
+      <c r="BD16" s="50" t="n"/>
+      <c r="BE16" s="45" t="n"/>
+      <c r="BF16" s="45" t="n"/>
+      <c r="BG16" s="50" t="n"/>
+      <c r="BH16" s="45" t="n"/>
+      <c r="BI16" s="45" t="n"/>
+      <c r="BJ16" s="50" t="n"/>
+      <c r="BK16" s="45" t="n"/>
+      <c r="BL16" s="45" t="n"/>
+      <c r="BM16" s="50" t="n"/>
+      <c r="BN16" s="45" t="n"/>
+      <c r="BO16" s="45" t="n"/>
+      <c r="BP16" s="50" t="n"/>
+      <c r="BQ16" s="45" t="n"/>
+      <c r="BR16" s="45" t="n"/>
+      <c r="BS16" s="45" t="n"/>
+      <c r="BT16" s="45" t="n"/>
+      <c r="BU16" s="45" t="n"/>
+      <c r="BV16" s="45" t="n"/>
+      <c r="BW16" s="45" t="n"/>
+      <c r="BX16" s="45" t="n"/>
+      <c r="BY16" s="45" t="n"/>
+      <c r="BZ16" s="45" t="n"/>
+      <c r="CA16" s="45" t="n"/>
+      <c r="CB16" s="45" t="n"/>
+      <c r="CC16" s="45" t="n"/>
+      <c r="CD16" s="46" t="n"/>
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="B17" s="44" t="n"/>
@@ -4273,47 +5444,78 @@
       <c r="H17" s="45" t="n"/>
       <c r="I17" s="45" t="n"/>
       <c r="J17" s="45" t="n"/>
-      <c r="K17" s="45" t="n"/>
-      <c r="L17" s="50" t="n"/>
+      <c r="K17" s="50" t="n"/>
+      <c r="L17" s="45" t="n"/>
       <c r="M17" s="45" t="n"/>
-      <c r="N17" s="45" t="n"/>
+      <c r="N17" s="50" t="n"/>
       <c r="O17" s="45" t="n"/>
       <c r="P17" s="45" t="n"/>
-      <c r="Q17" s="45" t="n"/>
+      <c r="Q17" s="50" t="n"/>
       <c r="R17" s="45" t="n"/>
       <c r="S17" s="45" t="n"/>
-      <c r="T17" s="45" t="n"/>
+      <c r="T17" s="50" t="n"/>
       <c r="U17" s="45" t="n"/>
       <c r="V17" s="45" t="n"/>
-      <c r="W17" s="45" t="n"/>
-      <c r="X17" s="50" t="n"/>
+      <c r="W17" s="50" t="n"/>
+      <c r="X17" s="45" t="n"/>
       <c r="Y17" s="45" t="n"/>
-      <c r="Z17" s="45" t="n"/>
+      <c r="Z17" s="50" t="n"/>
       <c r="AA17" s="45" t="n"/>
       <c r="AB17" s="45" t="n"/>
-      <c r="AC17" s="45" t="n"/>
+      <c r="AC17" s="50" t="n"/>
       <c r="AD17" s="45" t="n"/>
       <c r="AE17" s="45" t="n"/>
-      <c r="AF17" s="45" t="n"/>
+      <c r="AF17" s="50" t="n"/>
       <c r="AG17" s="45" t="n"/>
       <c r="AH17" s="45" t="n"/>
-      <c r="AI17" s="45" t="n"/>
-      <c r="AJ17" s="50" t="n"/>
+      <c r="AI17" s="50" t="n"/>
+      <c r="AJ17" s="45" t="n"/>
       <c r="AK17" s="45" t="n"/>
-      <c r="AL17" s="45" t="n"/>
+      <c r="AL17" s="50" t="n"/>
       <c r="AM17" s="45" t="n"/>
       <c r="AN17" s="45" t="n"/>
-      <c r="AO17" s="45" t="n"/>
+      <c r="AO17" s="50" t="n"/>
       <c r="AP17" s="45" t="n"/>
       <c r="AQ17" s="45" t="n"/>
-      <c r="AR17" s="45" t="n"/>
+      <c r="AR17" s="50" t="n"/>
       <c r="AS17" s="45" t="n"/>
       <c r="AT17" s="45" t="n"/>
-      <c r="AU17" s="45" t="n"/>
+      <c r="AU17" s="50" t="n"/>
       <c r="AV17" s="45" t="n"/>
       <c r="AW17" s="45" t="n"/>
-      <c r="AX17" s="45" t="n"/>
-      <c r="AY17" s="46" t="n"/>
+      <c r="AX17" s="50" t="n"/>
+      <c r="AY17" s="45" t="n"/>
+      <c r="AZ17" s="45" t="n"/>
+      <c r="BA17" s="50" t="n"/>
+      <c r="BB17" s="45" t="n"/>
+      <c r="BC17" s="45" t="n"/>
+      <c r="BD17" s="50" t="n"/>
+      <c r="BE17" s="45" t="n"/>
+      <c r="BF17" s="45" t="n"/>
+      <c r="BG17" s="50" t="n"/>
+      <c r="BH17" s="45" t="n"/>
+      <c r="BI17" s="45" t="n"/>
+      <c r="BJ17" s="50" t="n"/>
+      <c r="BK17" s="45" t="n"/>
+      <c r="BL17" s="45" t="n"/>
+      <c r="BM17" s="50" t="n"/>
+      <c r="BN17" s="45" t="n"/>
+      <c r="BO17" s="45" t="n"/>
+      <c r="BP17" s="50" t="n"/>
+      <c r="BQ17" s="45" t="n"/>
+      <c r="BR17" s="45" t="n"/>
+      <c r="BS17" s="45" t="n"/>
+      <c r="BT17" s="45" t="n"/>
+      <c r="BU17" s="45" t="n"/>
+      <c r="BV17" s="45" t="n"/>
+      <c r="BW17" s="45" t="n"/>
+      <c r="BX17" s="45" t="n"/>
+      <c r="BY17" s="45" t="n"/>
+      <c r="BZ17" s="45" t="n"/>
+      <c r="CA17" s="45" t="n"/>
+      <c r="CB17" s="45" t="n"/>
+      <c r="CC17" s="45" t="n"/>
+      <c r="CD17" s="46" t="n"/>
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="B18" s="44" t="n"/>
@@ -4325,47 +5527,78 @@
       <c r="H18" s="45" t="n"/>
       <c r="I18" s="45" t="n"/>
       <c r="J18" s="45" t="n"/>
-      <c r="K18" s="45" t="n"/>
-      <c r="L18" s="50" t="n"/>
+      <c r="K18" s="50" t="n"/>
+      <c r="L18" s="45" t="n"/>
       <c r="M18" s="45" t="n"/>
-      <c r="N18" s="45" t="n"/>
+      <c r="N18" s="50" t="n"/>
       <c r="O18" s="45" t="n"/>
       <c r="P18" s="45" t="n"/>
-      <c r="Q18" s="45" t="n"/>
+      <c r="Q18" s="50" t="n"/>
       <c r="R18" s="45" t="n"/>
       <c r="S18" s="45" t="n"/>
-      <c r="T18" s="45" t="n"/>
+      <c r="T18" s="50" t="n"/>
       <c r="U18" s="45" t="n"/>
       <c r="V18" s="45" t="n"/>
-      <c r="W18" s="45" t="n"/>
-      <c r="X18" s="50" t="n"/>
+      <c r="W18" s="50" t="n"/>
+      <c r="X18" s="45" t="n"/>
       <c r="Y18" s="45" t="n"/>
-      <c r="Z18" s="45" t="n"/>
+      <c r="Z18" s="50" t="n"/>
       <c r="AA18" s="45" t="n"/>
       <c r="AB18" s="45" t="n"/>
-      <c r="AC18" s="45" t="n"/>
+      <c r="AC18" s="50" t="n"/>
       <c r="AD18" s="45" t="n"/>
       <c r="AE18" s="45" t="n"/>
-      <c r="AF18" s="45" t="n"/>
+      <c r="AF18" s="50" t="n"/>
       <c r="AG18" s="45" t="n"/>
       <c r="AH18" s="45" t="n"/>
-      <c r="AI18" s="45" t="n"/>
-      <c r="AJ18" s="50" t="n"/>
+      <c r="AI18" s="50" t="n"/>
+      <c r="AJ18" s="45" t="n"/>
       <c r="AK18" s="45" t="n"/>
-      <c r="AL18" s="45" t="n"/>
+      <c r="AL18" s="50" t="n"/>
       <c r="AM18" s="45" t="n"/>
       <c r="AN18" s="45" t="n"/>
-      <c r="AO18" s="45" t="n"/>
+      <c r="AO18" s="50" t="n"/>
       <c r="AP18" s="45" t="n"/>
       <c r="AQ18" s="45" t="n"/>
-      <c r="AR18" s="45" t="n"/>
+      <c r="AR18" s="50" t="n"/>
       <c r="AS18" s="45" t="n"/>
       <c r="AT18" s="45" t="n"/>
-      <c r="AU18" s="45" t="n"/>
+      <c r="AU18" s="50" t="n"/>
       <c r="AV18" s="45" t="n"/>
       <c r="AW18" s="45" t="n"/>
-      <c r="AX18" s="45" t="n"/>
-      <c r="AY18" s="46" t="n"/>
+      <c r="AX18" s="50" t="n"/>
+      <c r="AY18" s="45" t="n"/>
+      <c r="AZ18" s="45" t="n"/>
+      <c r="BA18" s="50" t="n"/>
+      <c r="BB18" s="45" t="n"/>
+      <c r="BC18" s="45" t="n"/>
+      <c r="BD18" s="50" t="n"/>
+      <c r="BE18" s="45" t="n"/>
+      <c r="BF18" s="45" t="n"/>
+      <c r="BG18" s="50" t="n"/>
+      <c r="BH18" s="45" t="n"/>
+      <c r="BI18" s="45" t="n"/>
+      <c r="BJ18" s="50" t="n"/>
+      <c r="BK18" s="45" t="n"/>
+      <c r="BL18" s="45" t="n"/>
+      <c r="BM18" s="50" t="n"/>
+      <c r="BN18" s="45" t="n"/>
+      <c r="BO18" s="45" t="n"/>
+      <c r="BP18" s="50" t="n"/>
+      <c r="BQ18" s="45" t="n"/>
+      <c r="BR18" s="45" t="n"/>
+      <c r="BS18" s="45" t="n"/>
+      <c r="BT18" s="45" t="n"/>
+      <c r="BU18" s="45" t="n"/>
+      <c r="BV18" s="45" t="n"/>
+      <c r="BW18" s="45" t="n"/>
+      <c r="BX18" s="45" t="n"/>
+      <c r="BY18" s="45" t="n"/>
+      <c r="BZ18" s="45" t="n"/>
+      <c r="CA18" s="45" t="n"/>
+      <c r="CB18" s="45" t="n"/>
+      <c r="CC18" s="45" t="n"/>
+      <c r="CD18" s="46" t="n"/>
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="B19" s="44" t="n"/>
@@ -4377,47 +5610,78 @@
       <c r="H19" s="45" t="n"/>
       <c r="I19" s="45" t="n"/>
       <c r="J19" s="45" t="n"/>
-      <c r="K19" s="45" t="n"/>
-      <c r="L19" s="50" t="n"/>
+      <c r="K19" s="50" t="n"/>
+      <c r="L19" s="45" t="n"/>
       <c r="M19" s="45" t="n"/>
-      <c r="N19" s="45" t="n"/>
+      <c r="N19" s="50" t="n"/>
       <c r="O19" s="45" t="n"/>
       <c r="P19" s="45" t="n"/>
-      <c r="Q19" s="45" t="n"/>
+      <c r="Q19" s="50" t="n"/>
       <c r="R19" s="45" t="n"/>
       <c r="S19" s="45" t="n"/>
-      <c r="T19" s="45" t="n"/>
+      <c r="T19" s="50" t="n"/>
       <c r="U19" s="45" t="n"/>
       <c r="V19" s="45" t="n"/>
-      <c r="W19" s="45" t="n"/>
-      <c r="X19" s="50" t="n"/>
+      <c r="W19" s="50" t="n"/>
+      <c r="X19" s="45" t="n"/>
       <c r="Y19" s="45" t="n"/>
-      <c r="Z19" s="45" t="n"/>
+      <c r="Z19" s="50" t="n"/>
       <c r="AA19" s="45" t="n"/>
       <c r="AB19" s="45" t="n"/>
-      <c r="AC19" s="45" t="n"/>
+      <c r="AC19" s="50" t="n"/>
       <c r="AD19" s="45" t="n"/>
       <c r="AE19" s="45" t="n"/>
-      <c r="AF19" s="45" t="n"/>
+      <c r="AF19" s="50" t="n"/>
       <c r="AG19" s="45" t="n"/>
       <c r="AH19" s="45" t="n"/>
-      <c r="AI19" s="45" t="n"/>
-      <c r="AJ19" s="50" t="n"/>
+      <c r="AI19" s="50" t="n"/>
+      <c r="AJ19" s="45" t="n"/>
       <c r="AK19" s="45" t="n"/>
-      <c r="AL19" s="45" t="n"/>
+      <c r="AL19" s="50" t="n"/>
       <c r="AM19" s="45" t="n"/>
       <c r="AN19" s="45" t="n"/>
-      <c r="AO19" s="45" t="n"/>
+      <c r="AO19" s="50" t="n"/>
       <c r="AP19" s="45" t="n"/>
       <c r="AQ19" s="45" t="n"/>
-      <c r="AR19" s="45" t="n"/>
+      <c r="AR19" s="50" t="n"/>
       <c r="AS19" s="45" t="n"/>
       <c r="AT19" s="45" t="n"/>
-      <c r="AU19" s="45" t="n"/>
+      <c r="AU19" s="50" t="n"/>
       <c r="AV19" s="45" t="n"/>
       <c r="AW19" s="45" t="n"/>
-      <c r="AX19" s="45" t="n"/>
-      <c r="AY19" s="46" t="n"/>
+      <c r="AX19" s="50" t="n"/>
+      <c r="AY19" s="45" t="n"/>
+      <c r="AZ19" s="45" t="n"/>
+      <c r="BA19" s="50" t="n"/>
+      <c r="BB19" s="45" t="n"/>
+      <c r="BC19" s="45" t="n"/>
+      <c r="BD19" s="50" t="n"/>
+      <c r="BE19" s="45" t="n"/>
+      <c r="BF19" s="45" t="n"/>
+      <c r="BG19" s="50" t="n"/>
+      <c r="BH19" s="45" t="n"/>
+      <c r="BI19" s="45" t="n"/>
+      <c r="BJ19" s="50" t="n"/>
+      <c r="BK19" s="45" t="n"/>
+      <c r="BL19" s="45" t="n"/>
+      <c r="BM19" s="50" t="n"/>
+      <c r="BN19" s="45" t="n"/>
+      <c r="BO19" s="45" t="n"/>
+      <c r="BP19" s="50" t="n"/>
+      <c r="BQ19" s="45" t="n"/>
+      <c r="BR19" s="45" t="n"/>
+      <c r="BS19" s="45" t="n"/>
+      <c r="BT19" s="45" t="n"/>
+      <c r="BU19" s="45" t="n"/>
+      <c r="BV19" s="45" t="n"/>
+      <c r="BW19" s="45" t="n"/>
+      <c r="BX19" s="45" t="n"/>
+      <c r="BY19" s="45" t="n"/>
+      <c r="BZ19" s="45" t="n"/>
+      <c r="CA19" s="45" t="n"/>
+      <c r="CB19" s="45" t="n"/>
+      <c r="CC19" s="45" t="n"/>
+      <c r="CD19" s="46" t="n"/>
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="B20" s="44" t="n"/>
@@ -4429,47 +5693,78 @@
       <c r="H20" s="45" t="n"/>
       <c r="I20" s="45" t="n"/>
       <c r="J20" s="45" t="n"/>
-      <c r="K20" s="45" t="n"/>
-      <c r="L20" s="50" t="n"/>
+      <c r="K20" s="50" t="n"/>
+      <c r="L20" s="45" t="n"/>
       <c r="M20" s="45" t="n"/>
-      <c r="N20" s="45" t="n"/>
+      <c r="N20" s="50" t="n"/>
       <c r="O20" s="45" t="n"/>
       <c r="P20" s="45" t="n"/>
-      <c r="Q20" s="45" t="n"/>
+      <c r="Q20" s="50" t="n"/>
       <c r="R20" s="45" t="n"/>
       <c r="S20" s="45" t="n"/>
-      <c r="T20" s="45" t="n"/>
+      <c r="T20" s="50" t="n"/>
       <c r="U20" s="45" t="n"/>
       <c r="V20" s="45" t="n"/>
-      <c r="W20" s="45" t="n"/>
-      <c r="X20" s="50" t="n"/>
+      <c r="W20" s="50" t="n"/>
+      <c r="X20" s="45" t="n"/>
       <c r="Y20" s="45" t="n"/>
-      <c r="Z20" s="45" t="n"/>
+      <c r="Z20" s="50" t="n"/>
       <c r="AA20" s="45" t="n"/>
       <c r="AB20" s="45" t="n"/>
-      <c r="AC20" s="45" t="n"/>
+      <c r="AC20" s="50" t="n"/>
       <c r="AD20" s="45" t="n"/>
       <c r="AE20" s="45" t="n"/>
-      <c r="AF20" s="45" t="n"/>
+      <c r="AF20" s="50" t="n"/>
       <c r="AG20" s="45" t="n"/>
       <c r="AH20" s="45" t="n"/>
-      <c r="AI20" s="45" t="n"/>
-      <c r="AJ20" s="50" t="n"/>
+      <c r="AI20" s="50" t="n"/>
+      <c r="AJ20" s="45" t="n"/>
       <c r="AK20" s="45" t="n"/>
-      <c r="AL20" s="45" t="n"/>
+      <c r="AL20" s="50" t="n"/>
       <c r="AM20" s="45" t="n"/>
       <c r="AN20" s="45" t="n"/>
-      <c r="AO20" s="45" t="n"/>
+      <c r="AO20" s="50" t="n"/>
       <c r="AP20" s="45" t="n"/>
       <c r="AQ20" s="45" t="n"/>
-      <c r="AR20" s="45" t="n"/>
+      <c r="AR20" s="50" t="n"/>
       <c r="AS20" s="45" t="n"/>
       <c r="AT20" s="45" t="n"/>
-      <c r="AU20" s="45" t="n"/>
+      <c r="AU20" s="50" t="n"/>
       <c r="AV20" s="45" t="n"/>
       <c r="AW20" s="45" t="n"/>
-      <c r="AX20" s="45" t="n"/>
-      <c r="AY20" s="46" t="n"/>
+      <c r="AX20" s="50" t="n"/>
+      <c r="AY20" s="45" t="n"/>
+      <c r="AZ20" s="45" t="n"/>
+      <c r="BA20" s="50" t="n"/>
+      <c r="BB20" s="45" t="n"/>
+      <c r="BC20" s="45" t="n"/>
+      <c r="BD20" s="50" t="n"/>
+      <c r="BE20" s="45" t="n"/>
+      <c r="BF20" s="45" t="n"/>
+      <c r="BG20" s="50" t="n"/>
+      <c r="BH20" s="45" t="n"/>
+      <c r="BI20" s="45" t="n"/>
+      <c r="BJ20" s="50" t="n"/>
+      <c r="BK20" s="45" t="n"/>
+      <c r="BL20" s="45" t="n"/>
+      <c r="BM20" s="50" t="n"/>
+      <c r="BN20" s="45" t="n"/>
+      <c r="BO20" s="45" t="n"/>
+      <c r="BP20" s="50" t="n"/>
+      <c r="BQ20" s="45" t="n"/>
+      <c r="BR20" s="45" t="n"/>
+      <c r="BS20" s="45" t="n"/>
+      <c r="BT20" s="45" t="n"/>
+      <c r="BU20" s="45" t="n"/>
+      <c r="BV20" s="45" t="n"/>
+      <c r="BW20" s="45" t="n"/>
+      <c r="BX20" s="45" t="n"/>
+      <c r="BY20" s="45" t="n"/>
+      <c r="BZ20" s="45" t="n"/>
+      <c r="CA20" s="45" t="n"/>
+      <c r="CB20" s="45" t="n"/>
+      <c r="CC20" s="45" t="n"/>
+      <c r="CD20" s="46" t="n"/>
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="B21" s="44" t="n"/>
@@ -4481,47 +5776,78 @@
       <c r="H21" s="45" t="n"/>
       <c r="I21" s="45" t="n"/>
       <c r="J21" s="45" t="n"/>
-      <c r="K21" s="45" t="n"/>
-      <c r="L21" s="50" t="n"/>
+      <c r="K21" s="50" t="n"/>
+      <c r="L21" s="45" t="n"/>
       <c r="M21" s="45" t="n"/>
-      <c r="N21" s="45" t="n"/>
+      <c r="N21" s="50" t="n"/>
       <c r="O21" s="45" t="n"/>
       <c r="P21" s="45" t="n"/>
-      <c r="Q21" s="45" t="n"/>
+      <c r="Q21" s="50" t="n"/>
       <c r="R21" s="45" t="n"/>
       <c r="S21" s="45" t="n"/>
-      <c r="T21" s="45" t="n"/>
+      <c r="T21" s="50" t="n"/>
       <c r="U21" s="45" t="n"/>
       <c r="V21" s="45" t="n"/>
-      <c r="W21" s="45" t="n"/>
-      <c r="X21" s="50" t="n"/>
+      <c r="W21" s="50" t="n"/>
+      <c r="X21" s="45" t="n"/>
       <c r="Y21" s="45" t="n"/>
-      <c r="Z21" s="45" t="n"/>
+      <c r="Z21" s="50" t="n"/>
       <c r="AA21" s="45" t="n"/>
       <c r="AB21" s="45" t="n"/>
-      <c r="AC21" s="45" t="n"/>
+      <c r="AC21" s="50" t="n"/>
       <c r="AD21" s="45" t="n"/>
       <c r="AE21" s="45" t="n"/>
-      <c r="AF21" s="45" t="n"/>
+      <c r="AF21" s="50" t="n"/>
       <c r="AG21" s="45" t="n"/>
       <c r="AH21" s="45" t="n"/>
-      <c r="AI21" s="45" t="n"/>
-      <c r="AJ21" s="50" t="n"/>
+      <c r="AI21" s="50" t="n"/>
+      <c r="AJ21" s="45" t="n"/>
       <c r="AK21" s="45" t="n"/>
-      <c r="AL21" s="45" t="n"/>
+      <c r="AL21" s="50" t="n"/>
       <c r="AM21" s="45" t="n"/>
       <c r="AN21" s="45" t="n"/>
-      <c r="AO21" s="45" t="n"/>
+      <c r="AO21" s="50" t="n"/>
       <c r="AP21" s="45" t="n"/>
       <c r="AQ21" s="45" t="n"/>
-      <c r="AR21" s="45" t="n"/>
+      <c r="AR21" s="50" t="n"/>
       <c r="AS21" s="45" t="n"/>
       <c r="AT21" s="45" t="n"/>
-      <c r="AU21" s="45" t="n"/>
+      <c r="AU21" s="50" t="n"/>
       <c r="AV21" s="45" t="n"/>
       <c r="AW21" s="45" t="n"/>
-      <c r="AX21" s="45" t="n"/>
-      <c r="AY21" s="46" t="n"/>
+      <c r="AX21" s="50" t="n"/>
+      <c r="AY21" s="45" t="n"/>
+      <c r="AZ21" s="45" t="n"/>
+      <c r="BA21" s="50" t="n"/>
+      <c r="BB21" s="45" t="n"/>
+      <c r="BC21" s="45" t="n"/>
+      <c r="BD21" s="50" t="n"/>
+      <c r="BE21" s="45" t="n"/>
+      <c r="BF21" s="45" t="n"/>
+      <c r="BG21" s="50" t="n"/>
+      <c r="BH21" s="45" t="n"/>
+      <c r="BI21" s="45" t="n"/>
+      <c r="BJ21" s="50" t="n"/>
+      <c r="BK21" s="45" t="n"/>
+      <c r="BL21" s="45" t="n"/>
+      <c r="BM21" s="50" t="n"/>
+      <c r="BN21" s="45" t="n"/>
+      <c r="BO21" s="45" t="n"/>
+      <c r="BP21" s="50" t="n"/>
+      <c r="BQ21" s="45" t="n"/>
+      <c r="BR21" s="45" t="n"/>
+      <c r="BS21" s="45" t="n"/>
+      <c r="BT21" s="45" t="n"/>
+      <c r="BU21" s="45" t="n"/>
+      <c r="BV21" s="45" t="n"/>
+      <c r="BW21" s="45" t="n"/>
+      <c r="BX21" s="45" t="n"/>
+      <c r="BY21" s="45" t="n"/>
+      <c r="BZ21" s="45" t="n"/>
+      <c r="CA21" s="45" t="n"/>
+      <c r="CB21" s="45" t="n"/>
+      <c r="CC21" s="45" t="n"/>
+      <c r="CD21" s="46" t="n"/>
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="B22" s="44" t="n"/>
@@ -4573,7 +5899,38 @@
       <c r="AV22" s="45" t="n"/>
       <c r="AW22" s="45" t="n"/>
       <c r="AX22" s="45" t="n"/>
-      <c r="AY22" s="46" t="n"/>
+      <c r="AY22" s="45" t="n"/>
+      <c r="AZ22" s="45" t="n"/>
+      <c r="BA22" s="45" t="n"/>
+      <c r="BB22" s="45" t="n"/>
+      <c r="BC22" s="45" t="n"/>
+      <c r="BD22" s="45" t="n"/>
+      <c r="BE22" s="45" t="n"/>
+      <c r="BF22" s="45" t="n"/>
+      <c r="BG22" s="45" t="n"/>
+      <c r="BH22" s="45" t="n"/>
+      <c r="BI22" s="45" t="n"/>
+      <c r="BJ22" s="45" t="n"/>
+      <c r="BK22" s="45" t="n"/>
+      <c r="BL22" s="45" t="n"/>
+      <c r="BM22" s="45" t="n"/>
+      <c r="BN22" s="45" t="n"/>
+      <c r="BO22" s="45" t="n"/>
+      <c r="BP22" s="45" t="n"/>
+      <c r="BQ22" s="45" t="n"/>
+      <c r="BR22" s="45" t="n"/>
+      <c r="BS22" s="45" t="n"/>
+      <c r="BT22" s="45" t="n"/>
+      <c r="BU22" s="45" t="n"/>
+      <c r="BV22" s="45" t="n"/>
+      <c r="BW22" s="45" t="n"/>
+      <c r="BX22" s="45" t="n"/>
+      <c r="BY22" s="45" t="n"/>
+      <c r="BZ22" s="45" t="n"/>
+      <c r="CA22" s="45" t="n"/>
+      <c r="CB22" s="45" t="n"/>
+      <c r="CC22" s="45" t="n"/>
+      <c r="CD22" s="46" t="n"/>
     </row>
     <row r="23" ht="15" customHeight="1">
       <c r="B23" s="44" t="n"/>
@@ -4625,9 +5982,40 @@
       <c r="AV23" s="45" t="n"/>
       <c r="AW23" s="45" t="n"/>
       <c r="AX23" s="45" t="n"/>
-      <c r="AY23" s="46" t="n"/>
-    </row>
-    <row r="24" ht="15" customHeight="1">
+      <c r="AY23" s="45" t="n"/>
+      <c r="AZ23" s="45" t="n"/>
+      <c r="BA23" s="45" t="n"/>
+      <c r="BB23" s="45" t="n"/>
+      <c r="BC23" s="45" t="n"/>
+      <c r="BD23" s="45" t="n"/>
+      <c r="BE23" s="45" t="n"/>
+      <c r="BF23" s="45" t="n"/>
+      <c r="BG23" s="45" t="n"/>
+      <c r="BH23" s="45" t="n"/>
+      <c r="BI23" s="45" t="n"/>
+      <c r="BJ23" s="45" t="n"/>
+      <c r="BK23" s="45" t="n"/>
+      <c r="BL23" s="45" t="n"/>
+      <c r="BM23" s="45" t="n"/>
+      <c r="BN23" s="45" t="n"/>
+      <c r="BO23" s="45" t="n"/>
+      <c r="BP23" s="45" t="n"/>
+      <c r="BQ23" s="45" t="n"/>
+      <c r="BR23" s="45" t="n"/>
+      <c r="BS23" s="45" t="n"/>
+      <c r="BT23" s="45" t="n"/>
+      <c r="BU23" s="45" t="n"/>
+      <c r="BV23" s="45" t="n"/>
+      <c r="BW23" s="45" t="n"/>
+      <c r="BX23" s="45" t="n"/>
+      <c r="BY23" s="45" t="n"/>
+      <c r="BZ23" s="45" t="n"/>
+      <c r="CA23" s="45" t="n"/>
+      <c r="CB23" s="45" t="n"/>
+      <c r="CC23" s="45" t="n"/>
+      <c r="CD23" s="46" t="n"/>
+    </row>
+    <row r="24" ht="60" customHeight="1">
       <c r="B24" s="44" t="n"/>
       <c r="C24" s="45" t="n"/>
       <c r="D24" s="45" t="n"/>
@@ -4636,48 +6024,139 @@
       <c r="G24" s="45" t="n"/>
       <c r="H24" s="45" t="n"/>
       <c r="I24" s="45" t="n"/>
-      <c r="J24" s="45" t="n"/>
+      <c r="J24" s="53">
+        <f>IFERROR('Makine Giris'!B5,"M1")</f>
+        <v/>
+      </c>
       <c r="K24" s="45" t="n"/>
       <c r="L24" s="45" t="n"/>
-      <c r="M24" s="45" t="n"/>
+      <c r="M24" s="53">
+        <f>IFERROR('Makine Giris'!B6,"M2")</f>
+        <v/>
+      </c>
       <c r="N24" s="45" t="n"/>
       <c r="O24" s="45" t="n"/>
-      <c r="P24" s="45" t="n"/>
+      <c r="P24" s="53">
+        <f>IFERROR('Makine Giris'!B7,"M3")</f>
+        <v/>
+      </c>
       <c r="Q24" s="45" t="n"/>
       <c r="R24" s="45" t="n"/>
-      <c r="S24" s="45" t="n"/>
+      <c r="S24" s="53">
+        <f>IFERROR('Makine Giris'!B8,"M4")</f>
+        <v/>
+      </c>
       <c r="T24" s="45" t="n"/>
       <c r="U24" s="45" t="n"/>
-      <c r="V24" s="45" t="n"/>
+      <c r="V24" s="53">
+        <f>IFERROR('Makine Giris'!B9,"M5")</f>
+        <v/>
+      </c>
       <c r="W24" s="45" t="n"/>
       <c r="X24" s="45" t="n"/>
-      <c r="Y24" s="45" t="n"/>
+      <c r="Y24" s="53">
+        <f>IFERROR('Makine Giris'!B10,"M6")</f>
+        <v/>
+      </c>
       <c r="Z24" s="45" t="n"/>
       <c r="AA24" s="45" t="n"/>
-      <c r="AB24" s="45" t="n"/>
+      <c r="AB24" s="53">
+        <f>IFERROR('Makine Giris'!B11,"M7")</f>
+        <v/>
+      </c>
       <c r="AC24" s="45" t="n"/>
       <c r="AD24" s="45" t="n"/>
-      <c r="AE24" s="45" t="n"/>
+      <c r="AE24" s="53">
+        <f>IFERROR('Makine Giris'!B12,"M8")</f>
+        <v/>
+      </c>
       <c r="AF24" s="45" t="n"/>
       <c r="AG24" s="45" t="n"/>
-      <c r="AH24" s="45" t="n"/>
+      <c r="AH24" s="53">
+        <f>IFERROR('Makine Giris'!B13,"M9")</f>
+        <v/>
+      </c>
       <c r="AI24" s="45" t="n"/>
       <c r="AJ24" s="45" t="n"/>
-      <c r="AK24" s="45" t="n"/>
+      <c r="AK24" s="53">
+        <f>IFERROR('Makine Giris'!B14,"M10")</f>
+        <v/>
+      </c>
       <c r="AL24" s="45" t="n"/>
       <c r="AM24" s="45" t="n"/>
-      <c r="AN24" s="45" t="n"/>
+      <c r="AN24" s="53">
+        <f>IFERROR('Makine Giris'!B15,"M11")</f>
+        <v/>
+      </c>
       <c r="AO24" s="45" t="n"/>
       <c r="AP24" s="45" t="n"/>
-      <c r="AQ24" s="45" t="n"/>
+      <c r="AQ24" s="53">
+        <f>IFERROR('Makine Giris'!B16,"M12")</f>
+        <v/>
+      </c>
       <c r="AR24" s="45" t="n"/>
       <c r="AS24" s="45" t="n"/>
-      <c r="AT24" s="45" t="n"/>
+      <c r="AT24" s="53">
+        <f>IFERROR('Makine Giris'!B17,"M13")</f>
+        <v/>
+      </c>
       <c r="AU24" s="45" t="n"/>
       <c r="AV24" s="45" t="n"/>
-      <c r="AW24" s="45" t="n"/>
+      <c r="AW24" s="53">
+        <f>IFERROR('Makine Giris'!B18,"M14")</f>
+        <v/>
+      </c>
       <c r="AX24" s="45" t="n"/>
-      <c r="AY24" s="46" t="n"/>
+      <c r="AY24" s="45" t="n"/>
+      <c r="AZ24" s="53">
+        <f>IFERROR('Makine Giris'!B19,"M15")</f>
+        <v/>
+      </c>
+      <c r="BA24" s="45" t="n"/>
+      <c r="BB24" s="45" t="n"/>
+      <c r="BC24" s="53">
+        <f>IFERROR('Makine Giris'!B20,"M16")</f>
+        <v/>
+      </c>
+      <c r="BD24" s="45" t="n"/>
+      <c r="BE24" s="45" t="n"/>
+      <c r="BF24" s="53">
+        <f>IFERROR('Makine Giris'!B21,"M17")</f>
+        <v/>
+      </c>
+      <c r="BG24" s="45" t="n"/>
+      <c r="BH24" s="45" t="n"/>
+      <c r="BI24" s="53">
+        <f>IFERROR('Makine Giris'!B22,"M18")</f>
+        <v/>
+      </c>
+      <c r="BJ24" s="45" t="n"/>
+      <c r="BK24" s="45" t="n"/>
+      <c r="BL24" s="53">
+        <f>IFERROR('Makine Giris'!B23,"M19")</f>
+        <v/>
+      </c>
+      <c r="BM24" s="45" t="n"/>
+      <c r="BN24" s="45" t="n"/>
+      <c r="BO24" s="53">
+        <f>IFERROR('Makine Giris'!B24,"M20")</f>
+        <v/>
+      </c>
+      <c r="BP24" s="45" t="n"/>
+      <c r="BQ24" s="45" t="n"/>
+      <c r="BR24" s="45" t="n"/>
+      <c r="BS24" s="45" t="n"/>
+      <c r="BT24" s="45" t="n"/>
+      <c r="BU24" s="45" t="n"/>
+      <c r="BV24" s="45" t="n"/>
+      <c r="BW24" s="45" t="n"/>
+      <c r="BX24" s="45" t="n"/>
+      <c r="BY24" s="45" t="n"/>
+      <c r="BZ24" s="45" t="n"/>
+      <c r="CA24" s="45" t="n"/>
+      <c r="CB24" s="45" t="n"/>
+      <c r="CC24" s="45" t="n"/>
+      <c r="CD24" s="46" t="n"/>
     </row>
     <row r="25" ht="15" customHeight="1">
       <c r="B25" s="44" t="n"/>
@@ -4688,14 +6167,11 @@
       <c r="G25" s="45" t="n"/>
       <c r="H25" s="45" t="n"/>
       <c r="I25" s="45" t="n"/>
-      <c r="J25" s="53">
-        <f>IFERROR('Makine Giris'!B5,"Makine 1")</f>
-        <v/>
-      </c>
-      <c r="K25" s="51" t="n"/>
-      <c r="L25" s="51" t="n"/>
-      <c r="M25" s="51" t="n"/>
-      <c r="N25" s="52" t="n"/>
+      <c r="J25" s="45" t="n"/>
+      <c r="K25" s="45" t="n"/>
+      <c r="L25" s="45" t="n"/>
+      <c r="M25" s="45" t="n"/>
+      <c r="N25" s="45" t="n"/>
       <c r="O25" s="45" t="n"/>
       <c r="P25" s="45" t="n"/>
       <c r="Q25" s="45" t="n"/>
@@ -4703,14 +6179,11 @@
       <c r="S25" s="45" t="n"/>
       <c r="T25" s="45" t="n"/>
       <c r="U25" s="45" t="n"/>
-      <c r="V25" s="53">
-        <f>IFERROR('Makine Giris'!B6,"Makine 2")</f>
-        <v/>
-      </c>
-      <c r="W25" s="51" t="n"/>
-      <c r="X25" s="51" t="n"/>
-      <c r="Y25" s="51" t="n"/>
-      <c r="Z25" s="52" t="n"/>
+      <c r="V25" s="45" t="n"/>
+      <c r="W25" s="45" t="n"/>
+      <c r="X25" s="45" t="n"/>
+      <c r="Y25" s="45" t="n"/>
+      <c r="Z25" s="45" t="n"/>
       <c r="AA25" s="45" t="n"/>
       <c r="AB25" s="45" t="n"/>
       <c r="AC25" s="45" t="n"/>
@@ -4718,14 +6191,11 @@
       <c r="AE25" s="45" t="n"/>
       <c r="AF25" s="45" t="n"/>
       <c r="AG25" s="45" t="n"/>
-      <c r="AH25" s="53">
-        <f>IFERROR('Makine Giris'!B7,"Makine 3")</f>
-        <v/>
-      </c>
-      <c r="AI25" s="51" t="n"/>
-      <c r="AJ25" s="51" t="n"/>
-      <c r="AK25" s="51" t="n"/>
-      <c r="AL25" s="52" t="n"/>
+      <c r="AH25" s="45" t="n"/>
+      <c r="AI25" s="45" t="n"/>
+      <c r="AJ25" s="45" t="n"/>
+      <c r="AK25" s="45" t="n"/>
+      <c r="AL25" s="45" t="n"/>
       <c r="AM25" s="45" t="n"/>
       <c r="AN25" s="45" t="n"/>
       <c r="AO25" s="45" t="n"/>
@@ -4738,7 +6208,38 @@
       <c r="AV25" s="45" t="n"/>
       <c r="AW25" s="45" t="n"/>
       <c r="AX25" s="45" t="n"/>
-      <c r="AY25" s="46" t="n"/>
+      <c r="AY25" s="45" t="n"/>
+      <c r="AZ25" s="45" t="n"/>
+      <c r="BA25" s="45" t="n"/>
+      <c r="BB25" s="45" t="n"/>
+      <c r="BC25" s="45" t="n"/>
+      <c r="BD25" s="45" t="n"/>
+      <c r="BE25" s="45" t="n"/>
+      <c r="BF25" s="45" t="n"/>
+      <c r="BG25" s="45" t="n"/>
+      <c r="BH25" s="45" t="n"/>
+      <c r="BI25" s="45" t="n"/>
+      <c r="BJ25" s="45" t="n"/>
+      <c r="BK25" s="45" t="n"/>
+      <c r="BL25" s="45" t="n"/>
+      <c r="BM25" s="45" t="n"/>
+      <c r="BN25" s="45" t="n"/>
+      <c r="BO25" s="45" t="n"/>
+      <c r="BP25" s="45" t="n"/>
+      <c r="BQ25" s="45" t="n"/>
+      <c r="BR25" s="45" t="n"/>
+      <c r="BS25" s="45" t="n"/>
+      <c r="BT25" s="45" t="n"/>
+      <c r="BU25" s="45" t="n"/>
+      <c r="BV25" s="45" t="n"/>
+      <c r="BW25" s="45" t="n"/>
+      <c r="BX25" s="45" t="n"/>
+      <c r="BY25" s="45" t="n"/>
+      <c r="BZ25" s="45" t="n"/>
+      <c r="CA25" s="45" t="n"/>
+      <c r="CB25" s="45" t="n"/>
+      <c r="CC25" s="45" t="n"/>
+      <c r="CD25" s="46" t="n"/>
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="B26" s="44" t="n"/>
@@ -4790,7 +6291,38 @@
       <c r="AV26" s="45" t="n"/>
       <c r="AW26" s="45" t="n"/>
       <c r="AX26" s="45" t="n"/>
-      <c r="AY26" s="46" t="n"/>
+      <c r="AY26" s="45" t="n"/>
+      <c r="AZ26" s="45" t="n"/>
+      <c r="BA26" s="45" t="n"/>
+      <c r="BB26" s="45" t="n"/>
+      <c r="BC26" s="45" t="n"/>
+      <c r="BD26" s="45" t="n"/>
+      <c r="BE26" s="45" t="n"/>
+      <c r="BF26" s="45" t="n"/>
+      <c r="BG26" s="45" t="n"/>
+      <c r="BH26" s="45" t="n"/>
+      <c r="BI26" s="45" t="n"/>
+      <c r="BJ26" s="45" t="n"/>
+      <c r="BK26" s="45" t="n"/>
+      <c r="BL26" s="45" t="n"/>
+      <c r="BM26" s="45" t="n"/>
+      <c r="BN26" s="45" t="n"/>
+      <c r="BO26" s="45" t="n"/>
+      <c r="BP26" s="45" t="n"/>
+      <c r="BQ26" s="45" t="n"/>
+      <c r="BR26" s="45" t="n"/>
+      <c r="BS26" s="45" t="n"/>
+      <c r="BT26" s="45" t="n"/>
+      <c r="BU26" s="45" t="n"/>
+      <c r="BV26" s="45" t="n"/>
+      <c r="BW26" s="45" t="n"/>
+      <c r="BX26" s="45" t="n"/>
+      <c r="BY26" s="45" t="n"/>
+      <c r="BZ26" s="45" t="n"/>
+      <c r="CA26" s="45" t="n"/>
+      <c r="CB26" s="45" t="n"/>
+      <c r="CC26" s="45" t="n"/>
+      <c r="CD26" s="46" t="n"/>
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="B27" s="44" t="n"/>
@@ -4842,7 +6374,38 @@
       <c r="AV27" s="45" t="n"/>
       <c r="AW27" s="45" t="n"/>
       <c r="AX27" s="45" t="n"/>
-      <c r="AY27" s="46" t="n"/>
+      <c r="AY27" s="45" t="n"/>
+      <c r="AZ27" s="45" t="n"/>
+      <c r="BA27" s="45" t="n"/>
+      <c r="BB27" s="45" t="n"/>
+      <c r="BC27" s="45" t="n"/>
+      <c r="BD27" s="45" t="n"/>
+      <c r="BE27" s="45" t="n"/>
+      <c r="BF27" s="45" t="n"/>
+      <c r="BG27" s="45" t="n"/>
+      <c r="BH27" s="45" t="n"/>
+      <c r="BI27" s="45" t="n"/>
+      <c r="BJ27" s="45" t="n"/>
+      <c r="BK27" s="45" t="n"/>
+      <c r="BL27" s="45" t="n"/>
+      <c r="BM27" s="45" t="n"/>
+      <c r="BN27" s="45" t="n"/>
+      <c r="BO27" s="45" t="n"/>
+      <c r="BP27" s="45" t="n"/>
+      <c r="BQ27" s="45" t="n"/>
+      <c r="BR27" s="45" t="n"/>
+      <c r="BS27" s="45" t="n"/>
+      <c r="BT27" s="45" t="n"/>
+      <c r="BU27" s="45" t="n"/>
+      <c r="BV27" s="45" t="n"/>
+      <c r="BW27" s="45" t="n"/>
+      <c r="BX27" s="45" t="n"/>
+      <c r="BY27" s="45" t="n"/>
+      <c r="BZ27" s="45" t="n"/>
+      <c r="CA27" s="45" t="n"/>
+      <c r="CB27" s="45" t="n"/>
+      <c r="CC27" s="45" t="n"/>
+      <c r="CD27" s="46" t="n"/>
     </row>
     <row r="28" ht="15" customHeight="1">
       <c r="B28" s="44" t="n"/>
@@ -4894,7 +6457,38 @@
       <c r="AV28" s="45" t="n"/>
       <c r="AW28" s="45" t="n"/>
       <c r="AX28" s="45" t="n"/>
-      <c r="AY28" s="46" t="n"/>
+      <c r="AY28" s="45" t="n"/>
+      <c r="AZ28" s="45" t="n"/>
+      <c r="BA28" s="45" t="n"/>
+      <c r="BB28" s="45" t="n"/>
+      <c r="BC28" s="45" t="n"/>
+      <c r="BD28" s="45" t="n"/>
+      <c r="BE28" s="45" t="n"/>
+      <c r="BF28" s="45" t="n"/>
+      <c r="BG28" s="45" t="n"/>
+      <c r="BH28" s="45" t="n"/>
+      <c r="BI28" s="45" t="n"/>
+      <c r="BJ28" s="45" t="n"/>
+      <c r="BK28" s="45" t="n"/>
+      <c r="BL28" s="45" t="n"/>
+      <c r="BM28" s="45" t="n"/>
+      <c r="BN28" s="45" t="n"/>
+      <c r="BO28" s="45" t="n"/>
+      <c r="BP28" s="45" t="n"/>
+      <c r="BQ28" s="45" t="n"/>
+      <c r="BR28" s="45" t="n"/>
+      <c r="BS28" s="45" t="n"/>
+      <c r="BT28" s="45" t="n"/>
+      <c r="BU28" s="45" t="n"/>
+      <c r="BV28" s="45" t="n"/>
+      <c r="BW28" s="45" t="n"/>
+      <c r="BX28" s="45" t="n"/>
+      <c r="BY28" s="45" t="n"/>
+      <c r="BZ28" s="45" t="n"/>
+      <c r="CA28" s="45" t="n"/>
+      <c r="CB28" s="45" t="n"/>
+      <c r="CC28" s="45" t="n"/>
+      <c r="CD28" s="46" t="n"/>
     </row>
     <row r="29" ht="15" customHeight="1">
       <c r="B29" s="44" t="n"/>
@@ -4946,7 +6540,38 @@
       <c r="AV29" s="45" t="n"/>
       <c r="AW29" s="45" t="n"/>
       <c r="AX29" s="45" t="n"/>
-      <c r="AY29" s="46" t="n"/>
+      <c r="AY29" s="45" t="n"/>
+      <c r="AZ29" s="45" t="n"/>
+      <c r="BA29" s="45" t="n"/>
+      <c r="BB29" s="45" t="n"/>
+      <c r="BC29" s="45" t="n"/>
+      <c r="BD29" s="45" t="n"/>
+      <c r="BE29" s="45" t="n"/>
+      <c r="BF29" s="45" t="n"/>
+      <c r="BG29" s="45" t="n"/>
+      <c r="BH29" s="45" t="n"/>
+      <c r="BI29" s="45" t="n"/>
+      <c r="BJ29" s="45" t="n"/>
+      <c r="BK29" s="45" t="n"/>
+      <c r="BL29" s="45" t="n"/>
+      <c r="BM29" s="45" t="n"/>
+      <c r="BN29" s="45" t="n"/>
+      <c r="BO29" s="45" t="n"/>
+      <c r="BP29" s="45" t="n"/>
+      <c r="BQ29" s="45" t="n"/>
+      <c r="BR29" s="45" t="n"/>
+      <c r="BS29" s="45" t="n"/>
+      <c r="BT29" s="45" t="n"/>
+      <c r="BU29" s="45" t="n"/>
+      <c r="BV29" s="45" t="n"/>
+      <c r="BW29" s="45" t="n"/>
+      <c r="BX29" s="45" t="n"/>
+      <c r="BY29" s="45" t="n"/>
+      <c r="BZ29" s="45" t="n"/>
+      <c r="CA29" s="45" t="n"/>
+      <c r="CB29" s="45" t="n"/>
+      <c r="CC29" s="45" t="n"/>
+      <c r="CD29" s="46" t="n"/>
     </row>
     <row r="30" ht="15" customHeight="1">
       <c r="B30" s="44" t="n"/>
@@ -4998,7 +6623,38 @@
       <c r="AV30" s="45" t="n"/>
       <c r="AW30" s="45" t="n"/>
       <c r="AX30" s="45" t="n"/>
-      <c r="AY30" s="46" t="n"/>
+      <c r="AY30" s="45" t="n"/>
+      <c r="AZ30" s="45" t="n"/>
+      <c r="BA30" s="45" t="n"/>
+      <c r="BB30" s="45" t="n"/>
+      <c r="BC30" s="45" t="n"/>
+      <c r="BD30" s="45" t="n"/>
+      <c r="BE30" s="45" t="n"/>
+      <c r="BF30" s="45" t="n"/>
+      <c r="BG30" s="45" t="n"/>
+      <c r="BH30" s="45" t="n"/>
+      <c r="BI30" s="45" t="n"/>
+      <c r="BJ30" s="45" t="n"/>
+      <c r="BK30" s="45" t="n"/>
+      <c r="BL30" s="45" t="n"/>
+      <c r="BM30" s="45" t="n"/>
+      <c r="BN30" s="45" t="n"/>
+      <c r="BO30" s="45" t="n"/>
+      <c r="BP30" s="45" t="n"/>
+      <c r="BQ30" s="45" t="n"/>
+      <c r="BR30" s="45" t="n"/>
+      <c r="BS30" s="45" t="n"/>
+      <c r="BT30" s="45" t="n"/>
+      <c r="BU30" s="45" t="n"/>
+      <c r="BV30" s="45" t="n"/>
+      <c r="BW30" s="45" t="n"/>
+      <c r="BX30" s="45" t="n"/>
+      <c r="BY30" s="45" t="n"/>
+      <c r="BZ30" s="45" t="n"/>
+      <c r="CA30" s="45" t="n"/>
+      <c r="CB30" s="45" t="n"/>
+      <c r="CC30" s="45" t="n"/>
+      <c r="CD30" s="46" t="n"/>
     </row>
     <row r="31" ht="15" customHeight="1">
       <c r="B31" s="44" t="n"/>
@@ -5050,7 +6706,38 @@
       <c r="AV31" s="45" t="n"/>
       <c r="AW31" s="45" t="n"/>
       <c r="AX31" s="45" t="n"/>
-      <c r="AY31" s="46" t="n"/>
+      <c r="AY31" s="45" t="n"/>
+      <c r="AZ31" s="45" t="n"/>
+      <c r="BA31" s="45" t="n"/>
+      <c r="BB31" s="45" t="n"/>
+      <c r="BC31" s="45" t="n"/>
+      <c r="BD31" s="45" t="n"/>
+      <c r="BE31" s="45" t="n"/>
+      <c r="BF31" s="45" t="n"/>
+      <c r="BG31" s="45" t="n"/>
+      <c r="BH31" s="45" t="n"/>
+      <c r="BI31" s="45" t="n"/>
+      <c r="BJ31" s="45" t="n"/>
+      <c r="BK31" s="45" t="n"/>
+      <c r="BL31" s="45" t="n"/>
+      <c r="BM31" s="45" t="n"/>
+      <c r="BN31" s="45" t="n"/>
+      <c r="BO31" s="45" t="n"/>
+      <c r="BP31" s="45" t="n"/>
+      <c r="BQ31" s="45" t="n"/>
+      <c r="BR31" s="45" t="n"/>
+      <c r="BS31" s="45" t="n"/>
+      <c r="BT31" s="45" t="n"/>
+      <c r="BU31" s="45" t="n"/>
+      <c r="BV31" s="45" t="n"/>
+      <c r="BW31" s="45" t="n"/>
+      <c r="BX31" s="45" t="n"/>
+      <c r="BY31" s="45" t="n"/>
+      <c r="BZ31" s="45" t="n"/>
+      <c r="CA31" s="45" t="n"/>
+      <c r="CB31" s="45" t="n"/>
+      <c r="CC31" s="45" t="n"/>
+      <c r="CD31" s="46" t="n"/>
     </row>
     <row r="32" ht="15" customHeight="1">
       <c r="B32" s="44" t="n"/>
@@ -5102,7 +6789,38 @@
       <c r="AV32" s="45" t="n"/>
       <c r="AW32" s="45" t="n"/>
       <c r="AX32" s="45" t="n"/>
-      <c r="AY32" s="46" t="n"/>
+      <c r="AY32" s="45" t="n"/>
+      <c r="AZ32" s="45" t="n"/>
+      <c r="BA32" s="45" t="n"/>
+      <c r="BB32" s="45" t="n"/>
+      <c r="BC32" s="45" t="n"/>
+      <c r="BD32" s="45" t="n"/>
+      <c r="BE32" s="45" t="n"/>
+      <c r="BF32" s="45" t="n"/>
+      <c r="BG32" s="45" t="n"/>
+      <c r="BH32" s="45" t="n"/>
+      <c r="BI32" s="45" t="n"/>
+      <c r="BJ32" s="45" t="n"/>
+      <c r="BK32" s="45" t="n"/>
+      <c r="BL32" s="45" t="n"/>
+      <c r="BM32" s="45" t="n"/>
+      <c r="BN32" s="45" t="n"/>
+      <c r="BO32" s="45" t="n"/>
+      <c r="BP32" s="45" t="n"/>
+      <c r="BQ32" s="45" t="n"/>
+      <c r="BR32" s="45" t="n"/>
+      <c r="BS32" s="45" t="n"/>
+      <c r="BT32" s="45" t="n"/>
+      <c r="BU32" s="45" t="n"/>
+      <c r="BV32" s="45" t="n"/>
+      <c r="BW32" s="45" t="n"/>
+      <c r="BX32" s="45" t="n"/>
+      <c r="BY32" s="45" t="n"/>
+      <c r="BZ32" s="45" t="n"/>
+      <c r="CA32" s="45" t="n"/>
+      <c r="CB32" s="45" t="n"/>
+      <c r="CC32" s="45" t="n"/>
+      <c r="CD32" s="46" t="n"/>
     </row>
     <row r="33" ht="15" customHeight="1">
       <c r="B33" s="44" t="n"/>
@@ -5154,7 +6872,38 @@
       <c r="AV33" s="45" t="n"/>
       <c r="AW33" s="45" t="n"/>
       <c r="AX33" s="45" t="n"/>
-      <c r="AY33" s="46" t="n"/>
+      <c r="AY33" s="45" t="n"/>
+      <c r="AZ33" s="45" t="n"/>
+      <c r="BA33" s="45" t="n"/>
+      <c r="BB33" s="45" t="n"/>
+      <c r="BC33" s="45" t="n"/>
+      <c r="BD33" s="45" t="n"/>
+      <c r="BE33" s="45" t="n"/>
+      <c r="BF33" s="45" t="n"/>
+      <c r="BG33" s="45" t="n"/>
+      <c r="BH33" s="45" t="n"/>
+      <c r="BI33" s="45" t="n"/>
+      <c r="BJ33" s="45" t="n"/>
+      <c r="BK33" s="45" t="n"/>
+      <c r="BL33" s="45" t="n"/>
+      <c r="BM33" s="45" t="n"/>
+      <c r="BN33" s="45" t="n"/>
+      <c r="BO33" s="45" t="n"/>
+      <c r="BP33" s="45" t="n"/>
+      <c r="BQ33" s="45" t="n"/>
+      <c r="BR33" s="45" t="n"/>
+      <c r="BS33" s="45" t="n"/>
+      <c r="BT33" s="45" t="n"/>
+      <c r="BU33" s="45" t="n"/>
+      <c r="BV33" s="45" t="n"/>
+      <c r="BW33" s="45" t="n"/>
+      <c r="BX33" s="45" t="n"/>
+      <c r="BY33" s="45" t="n"/>
+      <c r="BZ33" s="45" t="n"/>
+      <c r="CA33" s="45" t="n"/>
+      <c r="CB33" s="45" t="n"/>
+      <c r="CC33" s="45" t="n"/>
+      <c r="CD33" s="46" t="n"/>
     </row>
     <row r="34" ht="15" customHeight="1">
       <c r="B34" s="44" t="n"/>
@@ -5206,7 +6955,38 @@
       <c r="AV34" s="45" t="n"/>
       <c r="AW34" s="45" t="n"/>
       <c r="AX34" s="45" t="n"/>
-      <c r="AY34" s="46" t="n"/>
+      <c r="AY34" s="45" t="n"/>
+      <c r="AZ34" s="45" t="n"/>
+      <c r="BA34" s="45" t="n"/>
+      <c r="BB34" s="45" t="n"/>
+      <c r="BC34" s="45" t="n"/>
+      <c r="BD34" s="45" t="n"/>
+      <c r="BE34" s="45" t="n"/>
+      <c r="BF34" s="45" t="n"/>
+      <c r="BG34" s="45" t="n"/>
+      <c r="BH34" s="45" t="n"/>
+      <c r="BI34" s="45" t="n"/>
+      <c r="BJ34" s="45" t="n"/>
+      <c r="BK34" s="45" t="n"/>
+      <c r="BL34" s="45" t="n"/>
+      <c r="BM34" s="45" t="n"/>
+      <c r="BN34" s="45" t="n"/>
+      <c r="BO34" s="45" t="n"/>
+      <c r="BP34" s="45" t="n"/>
+      <c r="BQ34" s="45" t="n"/>
+      <c r="BR34" s="45" t="n"/>
+      <c r="BS34" s="45" t="n"/>
+      <c r="BT34" s="45" t="n"/>
+      <c r="BU34" s="45" t="n"/>
+      <c r="BV34" s="45" t="n"/>
+      <c r="BW34" s="45" t="n"/>
+      <c r="BX34" s="45" t="n"/>
+      <c r="BY34" s="45" t="n"/>
+      <c r="BZ34" s="45" t="n"/>
+      <c r="CA34" s="45" t="n"/>
+      <c r="CB34" s="45" t="n"/>
+      <c r="CC34" s="45" t="n"/>
+      <c r="CD34" s="46" t="n"/>
     </row>
     <row r="35" ht="15" customHeight="1">
       <c r="B35" s="44" t="n"/>
@@ -5258,7 +7038,38 @@
       <c r="AV35" s="45" t="n"/>
       <c r="AW35" s="45" t="n"/>
       <c r="AX35" s="45" t="n"/>
-      <c r="AY35" s="46" t="n"/>
+      <c r="AY35" s="45" t="n"/>
+      <c r="AZ35" s="45" t="n"/>
+      <c r="BA35" s="45" t="n"/>
+      <c r="BB35" s="45" t="n"/>
+      <c r="BC35" s="45" t="n"/>
+      <c r="BD35" s="45" t="n"/>
+      <c r="BE35" s="45" t="n"/>
+      <c r="BF35" s="45" t="n"/>
+      <c r="BG35" s="45" t="n"/>
+      <c r="BH35" s="45" t="n"/>
+      <c r="BI35" s="45" t="n"/>
+      <c r="BJ35" s="45" t="n"/>
+      <c r="BK35" s="45" t="n"/>
+      <c r="BL35" s="45" t="n"/>
+      <c r="BM35" s="45" t="n"/>
+      <c r="BN35" s="45" t="n"/>
+      <c r="BO35" s="45" t="n"/>
+      <c r="BP35" s="45" t="n"/>
+      <c r="BQ35" s="45" t="n"/>
+      <c r="BR35" s="45" t="n"/>
+      <c r="BS35" s="45" t="n"/>
+      <c r="BT35" s="45" t="n"/>
+      <c r="BU35" s="45" t="n"/>
+      <c r="BV35" s="45" t="n"/>
+      <c r="BW35" s="45" t="n"/>
+      <c r="BX35" s="45" t="n"/>
+      <c r="BY35" s="45" t="n"/>
+      <c r="BZ35" s="45" t="n"/>
+      <c r="CA35" s="45" t="n"/>
+      <c r="CB35" s="45" t="n"/>
+      <c r="CC35" s="45" t="n"/>
+      <c r="CD35" s="46" t="n"/>
     </row>
     <row r="36" ht="15" customHeight="1">
       <c r="B36" s="44" t="n"/>
@@ -5310,7 +7121,38 @@
       <c r="AV36" s="45" t="n"/>
       <c r="AW36" s="45" t="n"/>
       <c r="AX36" s="45" t="n"/>
-      <c r="AY36" s="46" t="n"/>
+      <c r="AY36" s="45" t="n"/>
+      <c r="AZ36" s="45" t="n"/>
+      <c r="BA36" s="45" t="n"/>
+      <c r="BB36" s="45" t="n"/>
+      <c r="BC36" s="45" t="n"/>
+      <c r="BD36" s="45" t="n"/>
+      <c r="BE36" s="45" t="n"/>
+      <c r="BF36" s="45" t="n"/>
+      <c r="BG36" s="45" t="n"/>
+      <c r="BH36" s="45" t="n"/>
+      <c r="BI36" s="45" t="n"/>
+      <c r="BJ36" s="45" t="n"/>
+      <c r="BK36" s="45" t="n"/>
+      <c r="BL36" s="45" t="n"/>
+      <c r="BM36" s="45" t="n"/>
+      <c r="BN36" s="45" t="n"/>
+      <c r="BO36" s="45" t="n"/>
+      <c r="BP36" s="45" t="n"/>
+      <c r="BQ36" s="45" t="n"/>
+      <c r="BR36" s="45" t="n"/>
+      <c r="BS36" s="45" t="n"/>
+      <c r="BT36" s="45" t="n"/>
+      <c r="BU36" s="45" t="n"/>
+      <c r="BV36" s="45" t="n"/>
+      <c r="BW36" s="45" t="n"/>
+      <c r="BX36" s="45" t="n"/>
+      <c r="BY36" s="45" t="n"/>
+      <c r="BZ36" s="45" t="n"/>
+      <c r="CA36" s="45" t="n"/>
+      <c r="CB36" s="45" t="n"/>
+      <c r="CC36" s="45" t="n"/>
+      <c r="CD36" s="46" t="n"/>
     </row>
     <row r="37" ht="15" customHeight="1">
       <c r="B37" s="44" t="n"/>
@@ -5362,7 +7204,38 @@
       <c r="AV37" s="45" t="n"/>
       <c r="AW37" s="45" t="n"/>
       <c r="AX37" s="45" t="n"/>
-      <c r="AY37" s="46" t="n"/>
+      <c r="AY37" s="45" t="n"/>
+      <c r="AZ37" s="45" t="n"/>
+      <c r="BA37" s="45" t="n"/>
+      <c r="BB37" s="45" t="n"/>
+      <c r="BC37" s="45" t="n"/>
+      <c r="BD37" s="45" t="n"/>
+      <c r="BE37" s="45" t="n"/>
+      <c r="BF37" s="45" t="n"/>
+      <c r="BG37" s="45" t="n"/>
+      <c r="BH37" s="45" t="n"/>
+      <c r="BI37" s="45" t="n"/>
+      <c r="BJ37" s="45" t="n"/>
+      <c r="BK37" s="45" t="n"/>
+      <c r="BL37" s="45" t="n"/>
+      <c r="BM37" s="45" t="n"/>
+      <c r="BN37" s="45" t="n"/>
+      <c r="BO37" s="45" t="n"/>
+      <c r="BP37" s="45" t="n"/>
+      <c r="BQ37" s="45" t="n"/>
+      <c r="BR37" s="45" t="n"/>
+      <c r="BS37" s="45" t="n"/>
+      <c r="BT37" s="45" t="n"/>
+      <c r="BU37" s="45" t="n"/>
+      <c r="BV37" s="45" t="n"/>
+      <c r="BW37" s="45" t="n"/>
+      <c r="BX37" s="45" t="n"/>
+      <c r="BY37" s="45" t="n"/>
+      <c r="BZ37" s="45" t="n"/>
+      <c r="CA37" s="45" t="n"/>
+      <c r="CB37" s="45" t="n"/>
+      <c r="CC37" s="45" t="n"/>
+      <c r="CD37" s="46" t="n"/>
     </row>
     <row r="38" ht="15" customHeight="1">
       <c r="B38" s="44" t="n"/>
@@ -5414,7 +7287,38 @@
       <c r="AV38" s="45" t="n"/>
       <c r="AW38" s="45" t="n"/>
       <c r="AX38" s="45" t="n"/>
-      <c r="AY38" s="46" t="n"/>
+      <c r="AY38" s="45" t="n"/>
+      <c r="AZ38" s="45" t="n"/>
+      <c r="BA38" s="45" t="n"/>
+      <c r="BB38" s="45" t="n"/>
+      <c r="BC38" s="45" t="n"/>
+      <c r="BD38" s="45" t="n"/>
+      <c r="BE38" s="45" t="n"/>
+      <c r="BF38" s="45" t="n"/>
+      <c r="BG38" s="45" t="n"/>
+      <c r="BH38" s="45" t="n"/>
+      <c r="BI38" s="45" t="n"/>
+      <c r="BJ38" s="45" t="n"/>
+      <c r="BK38" s="45" t="n"/>
+      <c r="BL38" s="45" t="n"/>
+      <c r="BM38" s="45" t="n"/>
+      <c r="BN38" s="45" t="n"/>
+      <c r="BO38" s="45" t="n"/>
+      <c r="BP38" s="45" t="n"/>
+      <c r="BQ38" s="45" t="n"/>
+      <c r="BR38" s="45" t="n"/>
+      <c r="BS38" s="45" t="n"/>
+      <c r="BT38" s="45" t="n"/>
+      <c r="BU38" s="45" t="n"/>
+      <c r="BV38" s="45" t="n"/>
+      <c r="BW38" s="45" t="n"/>
+      <c r="BX38" s="45" t="n"/>
+      <c r="BY38" s="45" t="n"/>
+      <c r="BZ38" s="45" t="n"/>
+      <c r="CA38" s="45" t="n"/>
+      <c r="CB38" s="45" t="n"/>
+      <c r="CC38" s="45" t="n"/>
+      <c r="CD38" s="46" t="n"/>
     </row>
     <row r="39" ht="15" customHeight="1">
       <c r="B39" s="44" t="n"/>
@@ -5466,7 +7370,38 @@
       <c r="AV39" s="45" t="n"/>
       <c r="AW39" s="45" t="n"/>
       <c r="AX39" s="45" t="n"/>
-      <c r="AY39" s="46" t="n"/>
+      <c r="AY39" s="45" t="n"/>
+      <c r="AZ39" s="45" t="n"/>
+      <c r="BA39" s="45" t="n"/>
+      <c r="BB39" s="45" t="n"/>
+      <c r="BC39" s="45" t="n"/>
+      <c r="BD39" s="45" t="n"/>
+      <c r="BE39" s="45" t="n"/>
+      <c r="BF39" s="45" t="n"/>
+      <c r="BG39" s="45" t="n"/>
+      <c r="BH39" s="45" t="n"/>
+      <c r="BI39" s="45" t="n"/>
+      <c r="BJ39" s="45" t="n"/>
+      <c r="BK39" s="45" t="n"/>
+      <c r="BL39" s="45" t="n"/>
+      <c r="BM39" s="45" t="n"/>
+      <c r="BN39" s="45" t="n"/>
+      <c r="BO39" s="45" t="n"/>
+      <c r="BP39" s="45" t="n"/>
+      <c r="BQ39" s="45" t="n"/>
+      <c r="BR39" s="45" t="n"/>
+      <c r="BS39" s="45" t="n"/>
+      <c r="BT39" s="45" t="n"/>
+      <c r="BU39" s="45" t="n"/>
+      <c r="BV39" s="45" t="n"/>
+      <c r="BW39" s="45" t="n"/>
+      <c r="BX39" s="45" t="n"/>
+      <c r="BY39" s="45" t="n"/>
+      <c r="BZ39" s="45" t="n"/>
+      <c r="CA39" s="45" t="n"/>
+      <c r="CB39" s="45" t="n"/>
+      <c r="CC39" s="45" t="n"/>
+      <c r="CD39" s="46" t="n"/>
     </row>
     <row r="40" ht="15" customHeight="1">
       <c r="B40" s="44" t="n"/>
@@ -5518,7 +7453,38 @@
       <c r="AV40" s="45" t="n"/>
       <c r="AW40" s="45" t="n"/>
       <c r="AX40" s="45" t="n"/>
-      <c r="AY40" s="46" t="n"/>
+      <c r="AY40" s="45" t="n"/>
+      <c r="AZ40" s="45" t="n"/>
+      <c r="BA40" s="45" t="n"/>
+      <c r="BB40" s="45" t="n"/>
+      <c r="BC40" s="45" t="n"/>
+      <c r="BD40" s="45" t="n"/>
+      <c r="BE40" s="45" t="n"/>
+      <c r="BF40" s="45" t="n"/>
+      <c r="BG40" s="45" t="n"/>
+      <c r="BH40" s="45" t="n"/>
+      <c r="BI40" s="45" t="n"/>
+      <c r="BJ40" s="45" t="n"/>
+      <c r="BK40" s="45" t="n"/>
+      <c r="BL40" s="45" t="n"/>
+      <c r="BM40" s="45" t="n"/>
+      <c r="BN40" s="45" t="n"/>
+      <c r="BO40" s="45" t="n"/>
+      <c r="BP40" s="45" t="n"/>
+      <c r="BQ40" s="45" t="n"/>
+      <c r="BR40" s="45" t="n"/>
+      <c r="BS40" s="45" t="n"/>
+      <c r="BT40" s="45" t="n"/>
+      <c r="BU40" s="45" t="n"/>
+      <c r="BV40" s="45" t="n"/>
+      <c r="BW40" s="45" t="n"/>
+      <c r="BX40" s="45" t="n"/>
+      <c r="BY40" s="45" t="n"/>
+      <c r="BZ40" s="45" t="n"/>
+      <c r="CA40" s="45" t="n"/>
+      <c r="CB40" s="45" t="n"/>
+      <c r="CC40" s="45" t="n"/>
+      <c r="CD40" s="46" t="n"/>
     </row>
     <row r="41" ht="15" customHeight="1">
       <c r="B41" s="44" t="n"/>
@@ -5570,7 +7536,38 @@
       <c r="AV41" s="45" t="n"/>
       <c r="AW41" s="45" t="n"/>
       <c r="AX41" s="45" t="n"/>
-      <c r="AY41" s="46" t="n"/>
+      <c r="AY41" s="45" t="n"/>
+      <c r="AZ41" s="45" t="n"/>
+      <c r="BA41" s="45" t="n"/>
+      <c r="BB41" s="45" t="n"/>
+      <c r="BC41" s="45" t="n"/>
+      <c r="BD41" s="45" t="n"/>
+      <c r="BE41" s="45" t="n"/>
+      <c r="BF41" s="45" t="n"/>
+      <c r="BG41" s="45" t="n"/>
+      <c r="BH41" s="45" t="n"/>
+      <c r="BI41" s="45" t="n"/>
+      <c r="BJ41" s="45" t="n"/>
+      <c r="BK41" s="45" t="n"/>
+      <c r="BL41" s="45" t="n"/>
+      <c r="BM41" s="45" t="n"/>
+      <c r="BN41" s="45" t="n"/>
+      <c r="BO41" s="45" t="n"/>
+      <c r="BP41" s="45" t="n"/>
+      <c r="BQ41" s="45" t="n"/>
+      <c r="BR41" s="45" t="n"/>
+      <c r="BS41" s="45" t="n"/>
+      <c r="BT41" s="45" t="n"/>
+      <c r="BU41" s="45" t="n"/>
+      <c r="BV41" s="45" t="n"/>
+      <c r="BW41" s="45" t="n"/>
+      <c r="BX41" s="45" t="n"/>
+      <c r="BY41" s="45" t="n"/>
+      <c r="BZ41" s="45" t="n"/>
+      <c r="CA41" s="45" t="n"/>
+      <c r="CB41" s="45" t="n"/>
+      <c r="CC41" s="45" t="n"/>
+      <c r="CD41" s="46" t="n"/>
     </row>
     <row r="42" ht="15" customHeight="1">
       <c r="B42" s="54" t="n"/>
@@ -5622,7 +7619,38 @@
       <c r="AV42" s="55" t="n"/>
       <c r="AW42" s="55" t="n"/>
       <c r="AX42" s="55" t="n"/>
-      <c r="AY42" s="56" t="n"/>
+      <c r="AY42" s="55" t="n"/>
+      <c r="AZ42" s="55" t="n"/>
+      <c r="BA42" s="55" t="n"/>
+      <c r="BB42" s="55" t="n"/>
+      <c r="BC42" s="55" t="n"/>
+      <c r="BD42" s="55" t="n"/>
+      <c r="BE42" s="55" t="n"/>
+      <c r="BF42" s="55" t="n"/>
+      <c r="BG42" s="55" t="n"/>
+      <c r="BH42" s="55" t="n"/>
+      <c r="BI42" s="55" t="n"/>
+      <c r="BJ42" s="55" t="n"/>
+      <c r="BK42" s="55" t="n"/>
+      <c r="BL42" s="55" t="n"/>
+      <c r="BM42" s="55" t="n"/>
+      <c r="BN42" s="55" t="n"/>
+      <c r="BO42" s="55" t="n"/>
+      <c r="BP42" s="55" t="n"/>
+      <c r="BQ42" s="55" t="n"/>
+      <c r="BR42" s="55" t="n"/>
+      <c r="BS42" s="55" t="n"/>
+      <c r="BT42" s="55" t="n"/>
+      <c r="BU42" s="55" t="n"/>
+      <c r="BV42" s="55" t="n"/>
+      <c r="BW42" s="55" t="n"/>
+      <c r="BX42" s="55" t="n"/>
+      <c r="BY42" s="55" t="n"/>
+      <c r="BZ42" s="55" t="n"/>
+      <c r="CA42" s="55" t="n"/>
+      <c r="CB42" s="55" t="n"/>
+      <c r="CC42" s="55" t="n"/>
+      <c r="CD42" s="56" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="23" t="inlineStr">
@@ -5697,21 +7725,18 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="12">
     <mergeCell ref="A1:T1"/>
     <mergeCell ref="A44:J44"/>
     <mergeCell ref="C48:J48"/>
-    <mergeCell ref="V25:Z25"/>
-    <mergeCell ref="J25:N25"/>
+    <mergeCell ref="C51:J51"/>
     <mergeCell ref="C46:J46"/>
     <mergeCell ref="C47:J47"/>
-    <mergeCell ref="C51:J51"/>
-    <mergeCell ref="AH25:AL25"/>
     <mergeCell ref="A53:T53"/>
     <mergeCell ref="C50:J50"/>
     <mergeCell ref="A2:T2"/>
     <mergeCell ref="C45:J45"/>
-    <mergeCell ref="AU11:AX11"/>
+    <mergeCell ref="BZ11:CC11"/>
     <mergeCell ref="C49:J49"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>